<commit_message>
Pre-fill February nómina data from PDF + fix prorrata default
Data from actual February 2026 nómina (MECALUX):
- Plus baja temperatura: 261.12€
- H. Desplazamiento: 216.47€
- H. Desplazamiento Festivo: 228.24€
- H. Extra Normal: 474.48€
- Dieta (exento): 764.16€
- Plus Actividad: 18.04€ (config default)
- Salario Convenio: 2,063.39€ (config)
- IRPF Enero: 18.11%, IRPF Febrero: 18.15%
- Prorrata SS base: 419.61€ (appears in Base CC of real nómina)

Expected February result: SS 238.61€, IRPF 592.01€, NETO 3,195.28€

https://claude.ai/code/session_01WLGGf5vt4LjNM5wLNiuW4q
</commit_message>
<xml_diff>
--- a/calculadora-nomina-v3.xlsx
+++ b/calculadora-nomina-v3.xlsx
@@ -44,7 +44,7 @@
     <t>Prorrata Pagas Extra (base SS)</t>
   </si>
   <si>
-    <t>← 0 si no aparece en tu nómina; pon el valor si aparece en base de cotización (ej: 419,61)</t>
+    <t>← aparece en la base CC de tu nómina (Base CC 3.207,47 = sujeto CC + 419,61). La paga extra se cobra por separado en jun/dic, pero este importe suma a la base de cotización cada mes.</t>
   </si>
   <si>
     <t>Plus Actividad (por defecto)</t>
@@ -1366,7 +1366,7 @@
         <v>8</v>
       </c>
       <c r="C7" s="6">
-        <v>0</v>
+        <v>419.61</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>9</v>
@@ -1760,10 +1760,10 @@
         <v>64</v>
       </c>
       <c r="D4" s="8">
+        <v>0.1811</v>
+      </c>
+      <c r="E4" s="8">
         <v>0.1815</v>
-      </c>
-      <c r="E4" s="8">
-        <f>Configuración!$C$18</f>
       </c>
       <c r="F4" s="8">
         <f>Configuración!$C$18</f>
@@ -2036,7 +2036,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="6">
-        <v>0</v>
+        <v>261.12</v>
       </c>
       <c r="F11" s="6">
         <v>0</v>
@@ -2177,7 +2177,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="6">
-        <v>0</v>
+        <v>216.47</v>
       </c>
       <c r="F14" s="6">
         <v>0</v>
@@ -2224,7 +2224,7 @@
         <v>0</v>
       </c>
       <c r="E15" s="6">
-        <v>0</v>
+        <v>228.24</v>
       </c>
       <c r="F15" s="6">
         <v>0</v>
@@ -2318,7 +2318,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="6">
-        <v>0</v>
+        <v>474.48</v>
       </c>
       <c r="F17" s="6">
         <v>0</v>
@@ -2450,7 +2450,7 @@
         <v>0</v>
       </c>
       <c r="E21" s="6">
-        <v>0</v>
+        <v>764.16</v>
       </c>
       <c r="F21" s="6">
         <v>0</v>

</xml_diff>

<commit_message>
Add annual bruto/neto summary: con variables vs sin variables
Four key figures at the bottom of the sheet:
- BRUTO ANUAL con variables (total devengado: salary + extras + exempt + extra pays)
- Bruto anual sin variables (base salary × 12 + extra pays only)
- NETO ANUAL con variables (total liquid received across year)
- Neto anual sin variables (base salary net × 12 + net extra pays)
- Difference rows showing how much the variable extras contribute

SS for the "sin variables" base uses simplified formula:
  SS = (salary×12 + prorrata×12) × (CC% + Des+FP% + MEI%)  [no HHEE]

https://claude.ai/code/session_01WLGGf5vt4LjNM5wLNiuW4q
</commit_message>
<xml_diff>
--- a/calculadora-nomina-v3.xlsx
+++ b/calculadora-nomina-v3.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="137">
   <si>
     <t>⚙️  CONFIGURACIÓN — Nómina 2026</t>
   </si>
@@ -405,6 +405,27 @@
   </si>
   <si>
     <t>⚠️  Celdas amarillas = editables  |  IRPF editable por mes (fila "IRPF %")  |  Art.7p requiere trabajo físico en el extranjero y país destino con IRPF equivalente; consulta con gestor  |  Paga extra ⭐ = normalmente junio y diciembre; ponla en la fila "Paga Extra €" del mes correspondiente</t>
+  </si>
+  <si>
+    <t>📊  RESUMEN ANUAL — Bruto y Neto total (con variables) vs Solo salario fijo (sin variables)</t>
+  </si>
+  <si>
+    <t>💰  BRUTO ANUAL con variables  (devengado total: salario + extras + exentos + pagas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Bruto anual sin variables  (solo salario × 12 + pagas extras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Extra bruto generado por variables</t>
+  </si>
+  <si>
+    <t>💳  NETO ANUAL con variables  (líquido total cobrado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Neto anual sin variables  (solo salario fijo neto × 12 + neto pagas extras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Extra neto generado por variables</t>
   </si>
 </sst>
 </file>
@@ -414,7 +435,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00 &quot;€&quot;"/>
   </numFmts>
-  <fonts count="41" x14ac:knownFonts="1">
+  <fonts count="47" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -636,6 +657,40 @@
       <b/>
       <color rgb="FFFFFF"/>
       <sz val="13"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFF"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="4338CA"/>
+      <sz val="14"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="64748B"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="0F172A"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="0F172A"/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="0F172A"/>
+      <sz val="14"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -759,7 +814,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -955,6 +1010,33 @@
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="164" fontId="40" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="42" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="43" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="44" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="46" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1658,7 +1740,7 @@
     <tabColor rgb="4338CA"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P63"/>
+  <dimension ref="A1:P73"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -3918,8 +4000,214 @@
       <c r="O63" s="10"/>
       <c r="P63" s="10"/>
     </row>
+    <row r="64" ht="10" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A64" s="2"/>
+      <c r="B64" s="2"/>
+      <c r="C64" s="2"/>
+      <c r="D64" s="2"/>
+      <c r="E64" s="2"/>
+      <c r="F64" s="2"/>
+      <c r="G64" s="2"/>
+      <c r="H64" s="2"/>
+      <c r="I64" s="2"/>
+      <c r="J64" s="2"/>
+      <c r="K64" s="2"/>
+      <c r="L64" s="2"/>
+      <c r="M64" s="2"/>
+      <c r="N64" s="2"/>
+      <c r="O64" s="2"/>
+      <c r="P64" s="2"/>
+    </row>
+    <row r="65" ht="24" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A65" s="69" t="s">
+        <v>130</v>
+      </c>
+      <c r="B65" s="69"/>
+      <c r="C65" s="69"/>
+      <c r="D65" s="69"/>
+      <c r="E65" s="69"/>
+      <c r="F65" s="69"/>
+      <c r="G65" s="69"/>
+      <c r="H65" s="69"/>
+      <c r="I65" s="69"/>
+      <c r="J65" s="69"/>
+      <c r="K65" s="69"/>
+      <c r="L65" s="69"/>
+      <c r="M65" s="69"/>
+      <c r="N65" s="69"/>
+      <c r="O65" s="69"/>
+      <c r="P65" s="69"/>
+    </row>
+    <row r="66" ht="30" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A66" s="70" t="s">
+        <v>131</v>
+      </c>
+      <c r="B66" s="70"/>
+      <c r="C66" s="70"/>
+      <c r="D66" s="70"/>
+      <c r="E66" s="70"/>
+      <c r="F66" s="70"/>
+      <c r="G66" s="70"/>
+      <c r="H66" s="70"/>
+      <c r="I66" s="70"/>
+      <c r="J66" s="70"/>
+      <c r="K66" s="70"/>
+      <c r="L66" s="70"/>
+      <c r="M66" s="70"/>
+      <c r="N66" s="70"/>
+      <c r="O66" s="70"/>
+      <c r="P66" s="71">
+        <f>SUM(D29:O29)+SUM(D31:O31)+SUM(D26:O26)</f>
+      </c>
+    </row>
+    <row r="67" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A67" s="72" t="s">
+        <v>132</v>
+      </c>
+      <c r="B67" s="72"/>
+      <c r="C67" s="72"/>
+      <c r="D67" s="72"/>
+      <c r="E67" s="72"/>
+      <c r="F67" s="72"/>
+      <c r="G67" s="72"/>
+      <c r="H67" s="72"/>
+      <c r="I67" s="72"/>
+      <c r="J67" s="72"/>
+      <c r="K67" s="72"/>
+      <c r="L67" s="72"/>
+      <c r="M67" s="72"/>
+      <c r="N67" s="72"/>
+      <c r="O67" s="72"/>
+      <c r="P67" s="73">
+        <f>Configuración!$C$5*12+SUM(D26:O26)</f>
+      </c>
+    </row>
+    <row r="68" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A68" s="74" t="s">
+        <v>133</v>
+      </c>
+      <c r="B68" s="74"/>
+      <c r="C68" s="74"/>
+      <c r="D68" s="74"/>
+      <c r="E68" s="74"/>
+      <c r="F68" s="74"/>
+      <c r="G68" s="74"/>
+      <c r="H68" s="74"/>
+      <c r="I68" s="74"/>
+      <c r="J68" s="74"/>
+      <c r="K68" s="74"/>
+      <c r="L68" s="74"/>
+      <c r="M68" s="74"/>
+      <c r="N68" s="74"/>
+      <c r="O68" s="74"/>
+      <c r="P68" s="75">
+        <f>(SUM(D29:O29)+SUM(D31:O31)+SUM(D26:O26))-(Configuración!$C$5*12+SUM(D26:O26))</f>
+      </c>
+    </row>
+    <row r="69" ht="3" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A69" s="20"/>
+      <c r="B69" s="20"/>
+      <c r="C69" s="20"/>
+      <c r="D69" s="20"/>
+      <c r="E69" s="20"/>
+      <c r="F69" s="20"/>
+      <c r="G69" s="20"/>
+      <c r="H69" s="20"/>
+      <c r="I69" s="20"/>
+      <c r="J69" s="20"/>
+      <c r="K69" s="20"/>
+      <c r="L69" s="20"/>
+      <c r="M69" s="20"/>
+      <c r="N69" s="20"/>
+      <c r="O69" s="20"/>
+      <c r="P69" s="20"/>
+    </row>
+    <row r="70" ht="30" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A70" s="76" t="s">
+        <v>134</v>
+      </c>
+      <c r="B70" s="76"/>
+      <c r="C70" s="76"/>
+      <c r="D70" s="76"/>
+      <c r="E70" s="76"/>
+      <c r="F70" s="76"/>
+      <c r="G70" s="76"/>
+      <c r="H70" s="76"/>
+      <c r="I70" s="76"/>
+      <c r="J70" s="76"/>
+      <c r="K70" s="76"/>
+      <c r="L70" s="76"/>
+      <c r="M70" s="76"/>
+      <c r="N70" s="76"/>
+      <c r="O70" s="76"/>
+      <c r="P70" s="77">
+        <f>SUM(D49:O49)</f>
+      </c>
+    </row>
+    <row r="71" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A71" s="72" t="s">
+        <v>135</v>
+      </c>
+      <c r="B71" s="72"/>
+      <c r="C71" s="72"/>
+      <c r="D71" s="72"/>
+      <c r="E71" s="72"/>
+      <c r="F71" s="72"/>
+      <c r="G71" s="72"/>
+      <c r="H71" s="72"/>
+      <c r="I71" s="72"/>
+      <c r="J71" s="72"/>
+      <c r="K71" s="72"/>
+      <c r="L71" s="72"/>
+      <c r="M71" s="72"/>
+      <c r="N71" s="72"/>
+      <c r="O71" s="72"/>
+      <c r="P71" s="73">
+        <f>Configuración!$C$5*12-(Configuración!$C$5*12+Configuración!$C$7*12)*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)-Configuración!$C$5*12*Configuración!$C$18+SUM(D45:O45)</f>
+      </c>
+    </row>
+    <row r="72" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A72" s="74" t="s">
+        <v>136</v>
+      </c>
+      <c r="B72" s="74"/>
+      <c r="C72" s="74"/>
+      <c r="D72" s="74"/>
+      <c r="E72" s="74"/>
+      <c r="F72" s="74"/>
+      <c r="G72" s="74"/>
+      <c r="H72" s="74"/>
+      <c r="I72" s="74"/>
+      <c r="J72" s="74"/>
+      <c r="K72" s="74"/>
+      <c r="L72" s="74"/>
+      <c r="M72" s="74"/>
+      <c r="N72" s="74"/>
+      <c r="O72" s="74"/>
+      <c r="P72" s="75">
+        <f>(SUM(D49:O49))-(Configuración!$C$5*12-(Configuración!$C$5*12+Configuración!$C$7*12)*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)-Configuración!$C$5*12*Configuración!$C$18+SUM(D45:O45))</f>
+      </c>
+    </row>
+    <row r="73" ht="8" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A73" s="2"/>
+      <c r="B73" s="2"/>
+      <c r="C73" s="2"/>
+      <c r="D73" s="2"/>
+      <c r="E73" s="2"/>
+      <c r="F73" s="2"/>
+      <c r="G73" s="2"/>
+      <c r="H73" s="2"/>
+      <c r="I73" s="2"/>
+      <c r="J73" s="2"/>
+      <c r="K73" s="2"/>
+      <c r="L73" s="2"/>
+      <c r="M73" s="2"/>
+      <c r="N73" s="2"/>
+      <c r="O73" s="2"/>
+      <c r="P73" s="2"/>
+    </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="39">
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A2:P2"/>
     <mergeCell ref="A5:P5"/>
@@ -3949,6 +4237,16 @@
     <mergeCell ref="N61:P61"/>
     <mergeCell ref="A62:P62"/>
     <mergeCell ref="A63:P63"/>
+    <mergeCell ref="A64:P64"/>
+    <mergeCell ref="A65:P65"/>
+    <mergeCell ref="A66:O66"/>
+    <mergeCell ref="A67:O67"/>
+    <mergeCell ref="A68:O68"/>
+    <mergeCell ref="A69:P69"/>
+    <mergeCell ref="A70:O70"/>
+    <mergeCell ref="A71:O71"/>
+    <mergeCell ref="A72:O72"/>
+    <mergeCell ref="A73:P73"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Fix annual summary: sin variables = pure base salary only, no extras
- "Sin variables" now means ONLY salario convenio × 12 (no paga extra,
  no hours, no desplazamiento, no exentos — nothing extra)
- "Con variables" = everything devengado (salary + variables + exempt + extra pays)
- Neto sin variables = base salary net × 12 only (SS and IRPF on base only)

https://claude.ai/code/session_01WLGGf5vt4LjNM5wLNiuW4q
</commit_message>
<xml_diff>
--- a/calculadora-nomina-v3.xlsx
+++ b/calculadora-nomina-v3.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="136">
   <si>
     <t>⚙️  CONFIGURACIÓN — Nómina 2026</t>
   </si>
@@ -410,22 +410,19 @@
     <t>📊  RESUMEN ANUAL — Bruto y Neto total (con variables) vs Solo salario fijo (sin variables)</t>
   </si>
   <si>
-    <t>💰  BRUTO ANUAL con variables  (devengado total: salario + extras + exentos + pagas)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">     Bruto anual sin variables  (solo salario × 12 + pagas extras)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">     Extra bruto generado por variables</t>
-  </si>
-  <si>
-    <t>💳  NETO ANUAL con variables  (líquido total cobrado)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">     Neto anual sin variables  (solo salario fijo neto × 12 + neto pagas extras)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">     Extra neto generado por variables</t>
+    <t>💰  BRUTO ANUAL con variables  (salario + variables + exentos + pagas extra)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Bruto anual sin variables  (solo salario convenio × 12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Diferencia por variables</t>
+  </si>
+  <si>
+    <t>💳  NETO ANUAL con variables  (líquido total: salario + variables + pagas extra)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Neto anual sin variables  (solo salario fijo neto × 12)</t>
   </si>
 </sst>
 </file>
@@ -4079,7 +4076,7 @@
       <c r="N67" s="72"/>
       <c r="O67" s="72"/>
       <c r="P67" s="73">
-        <f>Configuración!$C$5*12+SUM(D26:O26)</f>
+        <f>Configuración!$C$5*12</f>
       </c>
     </row>
     <row r="68" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
@@ -4101,7 +4098,7 @@
       <c r="N68" s="74"/>
       <c r="O68" s="74"/>
       <c r="P68" s="75">
-        <f>(SUM(D29:O29)+SUM(D31:O31)+SUM(D26:O26))-(Configuración!$C$5*12+SUM(D26:O26))</f>
+        <f>(SUM(D29:O29)+SUM(D31:O31)+SUM(D26:O26))-(Configuración!$C$5*12)</f>
       </c>
     </row>
     <row r="69" ht="3" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
@@ -4163,12 +4160,12 @@
       <c r="N71" s="72"/>
       <c r="O71" s="72"/>
       <c r="P71" s="73">
-        <f>Configuración!$C$5*12-(Configuración!$C$5*12+Configuración!$C$7*12)*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)-Configuración!$C$5*12*Configuración!$C$18+SUM(D45:O45)</f>
+        <f>Configuración!$C$5*12-(Configuración!$C$5*12+Configuración!$C$7*12)*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)-Configuración!$C$5*12*Configuración!$C$18</f>
       </c>
     </row>
     <row r="72" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" s="74" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B72" s="74"/>
       <c r="C72" s="74"/>
@@ -4185,7 +4182,7 @@
       <c r="N72" s="74"/>
       <c r="O72" s="74"/>
       <c r="P72" s="75">
-        <f>(SUM(D49:O49))-(Configuración!$C$5*12-(Configuración!$C$5*12+Configuración!$C$7*12)*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)-Configuración!$C$5*12*Configuración!$C$18+SUM(D45:O45))</f>
+        <f>(SUM(D49:O49))-(Configuración!$C$5*12-(Configuración!$C$5*12+Configuración!$C$7*12)*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)-Configuración!$C$5*12*Configuración!$C$18)</f>
       </c>
     </row>
     <row r="73" ht="8" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Switch variable inputs to quantities: user enters hours/days/km
All variable rows now accept counts (hours, days, km) instead of euros.
The sheet calculates euros automatically: cantidad × precio unitario (config).

Changes:
- Turnicidad/Nocturnidad/Plus frío/H.Disp etc: input horas/días → × config price
- Días fuera: input número de días → × bruto/día
- KM: input kilómetros → × 0.30€
- Bruto Sujeto formula updated: all qty rows × their config price
- HHEE formula updated: HEX×PHEX + HEXF×PHEXF
- Exentos formula: Dieta + Tiquets + KM×PKM
- Art.7p D7P row now auto-references DIAF (no double entry)
- Art.7p TOT7P uses qty×price for DES, DESF, DIAF
- Total column always shows annual euros (qty×price summed)
- "Sin variables" summary fixed: only base salary ×12, no pagas extra

Feb pre-fill updated to qty: Plus frío 16d, H.Desp.Fest 18h, H.Extra 24h

https://claude.ai/code/session_01WLGGf5vt4LjNM5wLNiuW4q
</commit_message>
<xml_diff>
--- a/calculadora-nomina-v3.xlsx
+++ b/calculadora-nomina-v3.xlsx
@@ -227,55 +227,55 @@
     <t>Plus Actividad €</t>
   </si>
   <si>
-    <t>Turnicidad €</t>
-  </si>
-  <si>
-    <t>Nocturnidad €</t>
-  </si>
-  <si>
-    <t>Plus frío / baja temp. €</t>
-  </si>
-  <si>
-    <t>H. Disponibilidad €</t>
-  </si>
-  <si>
-    <t>H. Disp. Festiva €</t>
-  </si>
-  <si>
-    <t>H. Desplazamiento €</t>
+    <t>Turnicidad (horas)</t>
+  </si>
+  <si>
+    <t>Nocturnidad (horas)</t>
+  </si>
+  <si>
+    <t>Plus frío / baja temp. (días)</t>
+  </si>
+  <si>
+    <t>H. Disponibilidad (horas)</t>
+  </si>
+  <si>
+    <t>H. Disp. Festiva (horas)</t>
+  </si>
+  <si>
+    <t>H. Desplazamiento (horas)</t>
   </si>
   <si>
     <t>CC + 7p</t>
   </si>
   <si>
-    <t>H. Desp. Festivo €</t>
-  </si>
-  <si>
-    <t>Días fuera €</t>
-  </si>
-  <si>
-    <t>H. Extra Normal €</t>
+    <t>H. Desp. Festivo (horas)</t>
+  </si>
+  <si>
+    <t>Días fuera (días)</t>
+  </si>
+  <si>
+    <t>H. Extra Normal (horas)</t>
   </si>
   <si>
     <t>HHEE + 7p</t>
   </si>
   <si>
-    <t>H. Extra Festiva €</t>
+    <t>H. Extra Festiva (horas)</t>
   </si>
   <si>
     <t>🟢  EXENTOS — No cotizan SS ni retienen IRPF</t>
   </si>
   <si>
-    <t>Dieta €</t>
+    <t>Dieta € (importe directo)</t>
   </si>
   <si>
     <t>EXENTO</t>
   </si>
   <si>
-    <t>Tiquets €</t>
-  </si>
-  <si>
-    <t>KM €</t>
+    <t>Tiquets € (importe directo)</t>
+  </si>
+  <si>
+    <t>KM (kilómetros)</t>
   </si>
   <si>
     <t>⭐  PAGA EXTRA — Normalmente junio y diciembre. Pon el importe bruto en esos meses.</t>
@@ -365,10 +365,10 @@
     <t>🌍  ARTÍCULO 7p — Renta trabajos en el extranjero (potencialmente exenta de IRPF hasta 60.100€/año)</t>
   </si>
   <si>
-    <t>Nº días fuera España (para 7p)</t>
-  </si>
-  <si>
-    <t>input 7p</t>
+    <t>Días fuera España (= fila Días fuera)</t>
+  </si>
+  <si>
+    <t>auto 7p</t>
   </si>
   <si>
     <t>Proporción salario días fuera</t>
@@ -880,6 +880,9 @@
     <xf numFmtId="164" fontId="15" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="4" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -973,10 +976,7 @@
     <xf numFmtId="0" fontId="16" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="15" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="36" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="36" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2017,44 +2017,44 @@
       <c r="C9" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="D9" s="6">
-        <v>0</v>
-      </c>
-      <c r="E9" s="6">
-        <v>0</v>
-      </c>
-      <c r="F9" s="6">
-        <v>0</v>
-      </c>
-      <c r="G9" s="6">
-        <v>0</v>
-      </c>
-      <c r="H9" s="6">
-        <v>0</v>
-      </c>
-      <c r="I9" s="6">
-        <v>0</v>
-      </c>
-      <c r="J9" s="6">
-        <v>0</v>
-      </c>
-      <c r="K9" s="6">
-        <v>0</v>
-      </c>
-      <c r="L9" s="6">
-        <v>0</v>
-      </c>
-      <c r="M9" s="6">
-        <v>0</v>
-      </c>
-      <c r="N9" s="6">
-        <v>0</v>
-      </c>
-      <c r="O9" s="6">
+      <c r="D9" s="26">
+        <v>0</v>
+      </c>
+      <c r="E9" s="26">
+        <v>0</v>
+      </c>
+      <c r="F9" s="26">
+        <v>0</v>
+      </c>
+      <c r="G9" s="26">
+        <v>0</v>
+      </c>
+      <c r="H9" s="26">
+        <v>0</v>
+      </c>
+      <c r="I9" s="26">
+        <v>0</v>
+      </c>
+      <c r="J9" s="26">
+        <v>0</v>
+      </c>
+      <c r="K9" s="26">
+        <v>0</v>
+      </c>
+      <c r="L9" s="26">
+        <v>0</v>
+      </c>
+      <c r="M9" s="26">
+        <v>0</v>
+      </c>
+      <c r="N9" s="26">
+        <v>0</v>
+      </c>
+      <c r="O9" s="26">
         <v>0</v>
       </c>
       <c r="P9" s="25">
-        <f>SUM(D9:O9)</f>
+        <f>SUM(D9:O9)*Configuración!$C$22</f>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
@@ -2064,44 +2064,44 @@
       <c r="C10" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="6">
-        <v>0</v>
-      </c>
-      <c r="E10" s="6">
-        <v>0</v>
-      </c>
-      <c r="F10" s="6">
-        <v>0</v>
-      </c>
-      <c r="G10" s="6">
-        <v>0</v>
-      </c>
-      <c r="H10" s="6">
-        <v>0</v>
-      </c>
-      <c r="I10" s="6">
-        <v>0</v>
-      </c>
-      <c r="J10" s="6">
-        <v>0</v>
-      </c>
-      <c r="K10" s="6">
-        <v>0</v>
-      </c>
-      <c r="L10" s="6">
-        <v>0</v>
-      </c>
-      <c r="M10" s="6">
-        <v>0</v>
-      </c>
-      <c r="N10" s="6">
-        <v>0</v>
-      </c>
-      <c r="O10" s="6">
+      <c r="D10" s="26">
+        <v>0</v>
+      </c>
+      <c r="E10" s="26">
+        <v>0</v>
+      </c>
+      <c r="F10" s="26">
+        <v>0</v>
+      </c>
+      <c r="G10" s="26">
+        <v>0</v>
+      </c>
+      <c r="H10" s="26">
+        <v>0</v>
+      </c>
+      <c r="I10" s="26">
+        <v>0</v>
+      </c>
+      <c r="J10" s="26">
+        <v>0</v>
+      </c>
+      <c r="K10" s="26">
+        <v>0</v>
+      </c>
+      <c r="L10" s="26">
+        <v>0</v>
+      </c>
+      <c r="M10" s="26">
+        <v>0</v>
+      </c>
+      <c r="N10" s="26">
+        <v>0</v>
+      </c>
+      <c r="O10" s="26">
         <v>0</v>
       </c>
       <c r="P10" s="25">
-        <f>SUM(D10:O10)</f>
+        <f>SUM(D10:O10)*Configuración!$C$23</f>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
@@ -2111,44 +2111,44 @@
       <c r="C11" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="D11" s="6">
-        <v>0</v>
-      </c>
-      <c r="E11" s="6">
-        <v>261.12</v>
-      </c>
-      <c r="F11" s="6">
-        <v>0</v>
-      </c>
-      <c r="G11" s="6">
-        <v>0</v>
-      </c>
-      <c r="H11" s="6">
-        <v>0</v>
-      </c>
-      <c r="I11" s="6">
-        <v>0</v>
-      </c>
-      <c r="J11" s="6">
-        <v>0</v>
-      </c>
-      <c r="K11" s="6">
-        <v>0</v>
-      </c>
-      <c r="L11" s="6">
-        <v>0</v>
-      </c>
-      <c r="M11" s="6">
-        <v>0</v>
-      </c>
-      <c r="N11" s="6">
-        <v>0</v>
-      </c>
-      <c r="O11" s="6">
+      <c r="D11" s="26">
+        <v>0</v>
+      </c>
+      <c r="E11" s="26">
+        <v>16</v>
+      </c>
+      <c r="F11" s="26">
+        <v>0</v>
+      </c>
+      <c r="G11" s="26">
+        <v>0</v>
+      </c>
+      <c r="H11" s="26">
+        <v>0</v>
+      </c>
+      <c r="I11" s="26">
+        <v>0</v>
+      </c>
+      <c r="J11" s="26">
+        <v>0</v>
+      </c>
+      <c r="K11" s="26">
+        <v>0</v>
+      </c>
+      <c r="L11" s="26">
+        <v>0</v>
+      </c>
+      <c r="M11" s="26">
+        <v>0</v>
+      </c>
+      <c r="N11" s="26">
+        <v>0</v>
+      </c>
+      <c r="O11" s="26">
         <v>0</v>
       </c>
       <c r="P11" s="25">
-        <f>SUM(D11:O11)</f>
+        <f>SUM(D11:O11)*Configuración!$C$24</f>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
@@ -2158,44 +2158,44 @@
       <c r="C12" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="D12" s="6">
-        <v>0</v>
-      </c>
-      <c r="E12" s="6">
-        <v>0</v>
-      </c>
-      <c r="F12" s="6">
-        <v>0</v>
-      </c>
-      <c r="G12" s="6">
-        <v>0</v>
-      </c>
-      <c r="H12" s="6">
-        <v>0</v>
-      </c>
-      <c r="I12" s="6">
-        <v>0</v>
-      </c>
-      <c r="J12" s="6">
-        <v>0</v>
-      </c>
-      <c r="K12" s="6">
-        <v>0</v>
-      </c>
-      <c r="L12" s="6">
-        <v>0</v>
-      </c>
-      <c r="M12" s="6">
-        <v>0</v>
-      </c>
-      <c r="N12" s="6">
-        <v>0</v>
-      </c>
-      <c r="O12" s="6">
+      <c r="D12" s="26">
+        <v>0</v>
+      </c>
+      <c r="E12" s="26">
+        <v>0</v>
+      </c>
+      <c r="F12" s="26">
+        <v>0</v>
+      </c>
+      <c r="G12" s="26">
+        <v>0</v>
+      </c>
+      <c r="H12" s="26">
+        <v>0</v>
+      </c>
+      <c r="I12" s="26">
+        <v>0</v>
+      </c>
+      <c r="J12" s="26">
+        <v>0</v>
+      </c>
+      <c r="K12" s="26">
+        <v>0</v>
+      </c>
+      <c r="L12" s="26">
+        <v>0</v>
+      </c>
+      <c r="M12" s="26">
+        <v>0</v>
+      </c>
+      <c r="N12" s="26">
+        <v>0</v>
+      </c>
+      <c r="O12" s="26">
         <v>0</v>
       </c>
       <c r="P12" s="25">
-        <f>SUM(D12:O12)</f>
+        <f>SUM(D12:O12)*Configuración!$C$25</f>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
@@ -2205,279 +2205,279 @@
       <c r="C13" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="D13" s="6">
-        <v>0</v>
-      </c>
-      <c r="E13" s="6">
-        <v>0</v>
-      </c>
-      <c r="F13" s="6">
-        <v>0</v>
-      </c>
-      <c r="G13" s="6">
-        <v>0</v>
-      </c>
-      <c r="H13" s="6">
-        <v>0</v>
-      </c>
-      <c r="I13" s="6">
-        <v>0</v>
-      </c>
-      <c r="J13" s="6">
-        <v>0</v>
-      </c>
-      <c r="K13" s="6">
-        <v>0</v>
-      </c>
-      <c r="L13" s="6">
-        <v>0</v>
-      </c>
-      <c r="M13" s="6">
-        <v>0</v>
-      </c>
-      <c r="N13" s="6">
-        <v>0</v>
-      </c>
-      <c r="O13" s="6">
+      <c r="D13" s="26">
+        <v>0</v>
+      </c>
+      <c r="E13" s="26">
+        <v>0</v>
+      </c>
+      <c r="F13" s="26">
+        <v>0</v>
+      </c>
+      <c r="G13" s="26">
+        <v>0</v>
+      </c>
+      <c r="H13" s="26">
+        <v>0</v>
+      </c>
+      <c r="I13" s="26">
+        <v>0</v>
+      </c>
+      <c r="J13" s="26">
+        <v>0</v>
+      </c>
+      <c r="K13" s="26">
+        <v>0</v>
+      </c>
+      <c r="L13" s="26">
+        <v>0</v>
+      </c>
+      <c r="M13" s="26">
+        <v>0</v>
+      </c>
+      <c r="N13" s="26">
+        <v>0</v>
+      </c>
+      <c r="O13" s="26">
         <v>0</v>
       </c>
       <c r="P13" s="25">
-        <f>SUM(D13:O13)</f>
+        <f>SUM(D13:O13)*Configuración!$C$26</f>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B14" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="C14" s="26" t="s">
+      <c r="C14" s="27" t="s">
         <v>76</v>
       </c>
-      <c r="D14" s="6">
-        <v>0</v>
-      </c>
-      <c r="E14" s="6">
-        <v>216.47</v>
-      </c>
-      <c r="F14" s="6">
-        <v>0</v>
-      </c>
-      <c r="G14" s="6">
-        <v>0</v>
-      </c>
-      <c r="H14" s="6">
-        <v>0</v>
-      </c>
-      <c r="I14" s="6">
-        <v>0</v>
-      </c>
-      <c r="J14" s="6">
-        <v>0</v>
-      </c>
-      <c r="K14" s="6">
-        <v>0</v>
-      </c>
-      <c r="L14" s="6">
-        <v>0</v>
-      </c>
-      <c r="M14" s="6">
-        <v>0</v>
-      </c>
-      <c r="N14" s="6">
-        <v>0</v>
-      </c>
-      <c r="O14" s="6">
+      <c r="D14" s="26">
+        <v>0</v>
+      </c>
+      <c r="E14" s="26">
+        <v>20.5</v>
+      </c>
+      <c r="F14" s="26">
+        <v>0</v>
+      </c>
+      <c r="G14" s="26">
+        <v>0</v>
+      </c>
+      <c r="H14" s="26">
+        <v>0</v>
+      </c>
+      <c r="I14" s="26">
+        <v>0</v>
+      </c>
+      <c r="J14" s="26">
+        <v>0</v>
+      </c>
+      <c r="K14" s="26">
+        <v>0</v>
+      </c>
+      <c r="L14" s="26">
+        <v>0</v>
+      </c>
+      <c r="M14" s="26">
+        <v>0</v>
+      </c>
+      <c r="N14" s="26">
+        <v>0</v>
+      </c>
+      <c r="O14" s="26">
         <v>0</v>
       </c>
       <c r="P14" s="25">
-        <f>SUM(D14:O14)</f>
+        <f>SUM(D14:O14)*Configuración!$C$27</f>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B15" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="C15" s="26" t="s">
+      <c r="C15" s="27" t="s">
         <v>76</v>
       </c>
-      <c r="D15" s="6">
-        <v>0</v>
-      </c>
-      <c r="E15" s="6">
-        <v>228.24</v>
-      </c>
-      <c r="F15" s="6">
-        <v>0</v>
-      </c>
-      <c r="G15" s="6">
-        <v>0</v>
-      </c>
-      <c r="H15" s="6">
-        <v>0</v>
-      </c>
-      <c r="I15" s="6">
-        <v>0</v>
-      </c>
-      <c r="J15" s="6">
-        <v>0</v>
-      </c>
-      <c r="K15" s="6">
-        <v>0</v>
-      </c>
-      <c r="L15" s="6">
-        <v>0</v>
-      </c>
-      <c r="M15" s="6">
-        <v>0</v>
-      </c>
-      <c r="N15" s="6">
-        <v>0</v>
-      </c>
-      <c r="O15" s="6">
+      <c r="D15" s="26">
+        <v>0</v>
+      </c>
+      <c r="E15" s="26">
+        <v>18</v>
+      </c>
+      <c r="F15" s="26">
+        <v>0</v>
+      </c>
+      <c r="G15" s="26">
+        <v>0</v>
+      </c>
+      <c r="H15" s="26">
+        <v>0</v>
+      </c>
+      <c r="I15" s="26">
+        <v>0</v>
+      </c>
+      <c r="J15" s="26">
+        <v>0</v>
+      </c>
+      <c r="K15" s="26">
+        <v>0</v>
+      </c>
+      <c r="L15" s="26">
+        <v>0</v>
+      </c>
+      <c r="M15" s="26">
+        <v>0</v>
+      </c>
+      <c r="N15" s="26">
+        <v>0</v>
+      </c>
+      <c r="O15" s="26">
         <v>0</v>
       </c>
       <c r="P15" s="25">
-        <f>SUM(D15:O15)</f>
+        <f>SUM(D15:O15)*Configuración!$C$28</f>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B16" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="C16" s="26" t="s">
+      <c r="C16" s="27" t="s">
         <v>76</v>
       </c>
-      <c r="D16" s="6">
-        <v>0</v>
-      </c>
-      <c r="E16" s="6">
-        <v>0</v>
-      </c>
-      <c r="F16" s="6">
-        <v>0</v>
-      </c>
-      <c r="G16" s="6">
-        <v>0</v>
-      </c>
-      <c r="H16" s="6">
-        <v>0</v>
-      </c>
-      <c r="I16" s="6">
-        <v>0</v>
-      </c>
-      <c r="J16" s="6">
-        <v>0</v>
-      </c>
-      <c r="K16" s="6">
-        <v>0</v>
-      </c>
-      <c r="L16" s="6">
-        <v>0</v>
-      </c>
-      <c r="M16" s="6">
-        <v>0</v>
-      </c>
-      <c r="N16" s="6">
-        <v>0</v>
-      </c>
-      <c r="O16" s="6">
+      <c r="D16" s="26">
+        <v>0</v>
+      </c>
+      <c r="E16" s="26">
+        <v>0</v>
+      </c>
+      <c r="F16" s="26">
+        <v>0</v>
+      </c>
+      <c r="G16" s="26">
+        <v>0</v>
+      </c>
+      <c r="H16" s="26">
+        <v>0</v>
+      </c>
+      <c r="I16" s="26">
+        <v>0</v>
+      </c>
+      <c r="J16" s="26">
+        <v>0</v>
+      </c>
+      <c r="K16" s="26">
+        <v>0</v>
+      </c>
+      <c r="L16" s="26">
+        <v>0</v>
+      </c>
+      <c r="M16" s="26">
+        <v>0</v>
+      </c>
+      <c r="N16" s="26">
+        <v>0</v>
+      </c>
+      <c r="O16" s="26">
         <v>0</v>
       </c>
       <c r="P16" s="25">
-        <f>SUM(D16:O16)</f>
+        <f>SUM(D16:O16)*Configuración!$C$31</f>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B17" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="C17" s="27" t="s">
+      <c r="C17" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="D17" s="6">
-        <v>0</v>
-      </c>
-      <c r="E17" s="6">
-        <v>474.48</v>
-      </c>
-      <c r="F17" s="6">
-        <v>0</v>
-      </c>
-      <c r="G17" s="6">
-        <v>0</v>
-      </c>
-      <c r="H17" s="6">
-        <v>0</v>
-      </c>
-      <c r="I17" s="6">
-        <v>0</v>
-      </c>
-      <c r="J17" s="6">
-        <v>0</v>
-      </c>
-      <c r="K17" s="6">
-        <v>0</v>
-      </c>
-      <c r="L17" s="6">
-        <v>0</v>
-      </c>
-      <c r="M17" s="6">
-        <v>0</v>
-      </c>
-      <c r="N17" s="6">
-        <v>0</v>
-      </c>
-      <c r="O17" s="6">
+      <c r="D17" s="26">
+        <v>0</v>
+      </c>
+      <c r="E17" s="26">
+        <v>24</v>
+      </c>
+      <c r="F17" s="26">
+        <v>0</v>
+      </c>
+      <c r="G17" s="26">
+        <v>0</v>
+      </c>
+      <c r="H17" s="26">
+        <v>0</v>
+      </c>
+      <c r="I17" s="26">
+        <v>0</v>
+      </c>
+      <c r="J17" s="26">
+        <v>0</v>
+      </c>
+      <c r="K17" s="26">
+        <v>0</v>
+      </c>
+      <c r="L17" s="26">
+        <v>0</v>
+      </c>
+      <c r="M17" s="26">
+        <v>0</v>
+      </c>
+      <c r="N17" s="26">
+        <v>0</v>
+      </c>
+      <c r="O17" s="26">
         <v>0</v>
       </c>
       <c r="P17" s="25">
-        <f>SUM(D17:O17)</f>
+        <f>SUM(D17:O17)*Configuración!$C$29</f>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B18" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="C18" s="27" t="s">
+      <c r="C18" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="D18" s="6">
-        <v>0</v>
-      </c>
-      <c r="E18" s="6">
-        <v>0</v>
-      </c>
-      <c r="F18" s="6">
-        <v>0</v>
-      </c>
-      <c r="G18" s="6">
-        <v>0</v>
-      </c>
-      <c r="H18" s="6">
-        <v>0</v>
-      </c>
-      <c r="I18" s="6">
-        <v>0</v>
-      </c>
-      <c r="J18" s="6">
-        <v>0</v>
-      </c>
-      <c r="K18" s="6">
-        <v>0</v>
-      </c>
-      <c r="L18" s="6">
-        <v>0</v>
-      </c>
-      <c r="M18" s="6">
-        <v>0</v>
-      </c>
-      <c r="N18" s="6">
-        <v>0</v>
-      </c>
-      <c r="O18" s="6">
+      <c r="D18" s="26">
+        <v>0</v>
+      </c>
+      <c r="E18" s="26">
+        <v>0</v>
+      </c>
+      <c r="F18" s="26">
+        <v>0</v>
+      </c>
+      <c r="G18" s="26">
+        <v>0</v>
+      </c>
+      <c r="H18" s="26">
+        <v>0</v>
+      </c>
+      <c r="I18" s="26">
+        <v>0</v>
+      </c>
+      <c r="J18" s="26">
+        <v>0</v>
+      </c>
+      <c r="K18" s="26">
+        <v>0</v>
+      </c>
+      <c r="L18" s="26">
+        <v>0</v>
+      </c>
+      <c r="M18" s="26">
+        <v>0</v>
+      </c>
+      <c r="N18" s="26">
+        <v>0</v>
+      </c>
+      <c r="O18" s="26">
         <v>0</v>
       </c>
       <c r="P18" s="25">
-        <f>SUM(D18:O18)</f>
+        <f>SUM(D18:O18)*Configuración!$C$30</f>
       </c>
     </row>
     <row r="19" ht="2" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
@@ -2499,30 +2499,30 @@
       <c r="P19" s="20"/>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A20" s="28" t="s">
+      <c r="A20" s="29" t="s">
         <v>82</v>
       </c>
-      <c r="B20" s="28"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="28"/>
-      <c r="F20" s="28"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="28"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="28"/>
-      <c r="K20" s="28"/>
-      <c r="L20" s="28"/>
-      <c r="M20" s="28"/>
-      <c r="N20" s="28"/>
-      <c r="O20" s="28"/>
-      <c r="P20" s="28"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="29"/>
+      <c r="I20" s="29"/>
+      <c r="J20" s="29"/>
+      <c r="K20" s="29"/>
+      <c r="L20" s="29"/>
+      <c r="M20" s="29"/>
+      <c r="N20" s="29"/>
+      <c r="O20" s="29"/>
+      <c r="P20" s="29"/>
     </row>
     <row r="21" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B21" s="29" t="s">
+      <c r="B21" s="30" t="s">
         <v>83</v>
       </c>
-      <c r="C21" s="30" t="s">
+      <c r="C21" s="31" t="s">
         <v>84</v>
       </c>
       <c r="D21" s="6">
@@ -2566,10 +2566,10 @@
       </c>
     </row>
     <row r="22" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B22" s="29" t="s">
+      <c r="B22" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="C22" s="30" t="s">
+      <c r="C22" s="31" t="s">
         <v>84</v>
       </c>
       <c r="D22" s="6">
@@ -2613,50 +2613,50 @@
       </c>
     </row>
     <row r="23" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B23" s="29" t="s">
+      <c r="B23" s="30" t="s">
         <v>86</v>
       </c>
-      <c r="C23" s="30" t="s">
+      <c r="C23" s="31" t="s">
         <v>84</v>
       </c>
-      <c r="D23" s="6">
-        <v>0</v>
-      </c>
-      <c r="E23" s="6">
-        <v>0</v>
-      </c>
-      <c r="F23" s="6">
-        <v>0</v>
-      </c>
-      <c r="G23" s="6">
-        <v>0</v>
-      </c>
-      <c r="H23" s="6">
-        <v>0</v>
-      </c>
-      <c r="I23" s="6">
-        <v>0</v>
-      </c>
-      <c r="J23" s="6">
-        <v>0</v>
-      </c>
-      <c r="K23" s="6">
-        <v>0</v>
-      </c>
-      <c r="L23" s="6">
-        <v>0</v>
-      </c>
-      <c r="M23" s="6">
-        <v>0</v>
-      </c>
-      <c r="N23" s="6">
-        <v>0</v>
-      </c>
-      <c r="O23" s="6">
+      <c r="D23" s="26">
+        <v>0</v>
+      </c>
+      <c r="E23" s="26">
+        <v>0</v>
+      </c>
+      <c r="F23" s="26">
+        <v>0</v>
+      </c>
+      <c r="G23" s="26">
+        <v>0</v>
+      </c>
+      <c r="H23" s="26">
+        <v>0</v>
+      </c>
+      <c r="I23" s="26">
+        <v>0</v>
+      </c>
+      <c r="J23" s="26">
+        <v>0</v>
+      </c>
+      <c r="K23" s="26">
+        <v>0</v>
+      </c>
+      <c r="L23" s="26">
+        <v>0</v>
+      </c>
+      <c r="M23" s="26">
+        <v>0</v>
+      </c>
+      <c r="N23" s="26">
+        <v>0</v>
+      </c>
+      <c r="O23" s="26">
         <v>0</v>
       </c>
       <c r="P23" s="25">
-        <f>SUM(D23:O23)</f>
+        <f>SUM(D23:O23)*Configuración!$C$32</f>
       </c>
     </row>
     <row r="24" ht="2" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
@@ -2678,30 +2678,30 @@
       <c r="P24" s="20"/>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A25" s="31" t="s">
+      <c r="A25" s="32" t="s">
         <v>87</v>
       </c>
-      <c r="B25" s="31"/>
-      <c r="C25" s="31"/>
-      <c r="D25" s="31"/>
-      <c r="E25" s="31"/>
-      <c r="F25" s="31"/>
-      <c r="G25" s="31"/>
-      <c r="H25" s="31"/>
-      <c r="I25" s="31"/>
-      <c r="J25" s="31"/>
-      <c r="K25" s="31"/>
-      <c r="L25" s="31"/>
-      <c r="M25" s="31"/>
-      <c r="N25" s="31"/>
-      <c r="O25" s="31"/>
-      <c r="P25" s="31"/>
+      <c r="B25" s="32"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="32"/>
+      <c r="K25" s="32"/>
+      <c r="L25" s="32"/>
+      <c r="M25" s="32"/>
+      <c r="N25" s="32"/>
+      <c r="O25" s="32"/>
+      <c r="P25" s="32"/>
     </row>
     <row r="26" ht="20" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B26" s="32" t="s">
+      <c r="B26" s="33" t="s">
         <v>88</v>
       </c>
-      <c r="C26" s="33" t="s">
+      <c r="C26" s="34" t="s">
         <v>89</v>
       </c>
       <c r="D26" s="6">
@@ -2783,141 +2783,141 @@
       <c r="P28" s="3"/>
     </row>
     <row r="29" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B29" s="34" t="s">
+      <c r="B29" s="35" t="s">
         <v>91</v>
       </c>
-      <c r="C29" s="35" t="s">
+      <c r="C29" s="36" t="s">
         <v>92</v>
       </c>
-      <c r="D29" s="36">
-        <f>D7+D8+D9+D10+D11+D12+D13+D14+D15+D16+D17+D18</f>
-      </c>
-      <c r="E29" s="36">
-        <f>E7+E8+E9+E10+E11+E12+E13+E14+E15+E16+E17+E18</f>
-      </c>
-      <c r="F29" s="36">
-        <f>F7+F8+F9+F10+F11+F12+F13+F14+F15+F16+F17+F18</f>
-      </c>
-      <c r="G29" s="36">
-        <f>G7+G8+G9+G10+G11+G12+G13+G14+G15+G16+G17+G18</f>
-      </c>
-      <c r="H29" s="36">
-        <f>H7+H8+H9+H10+H11+H12+H13+H14+H15+H16+H17+H18</f>
-      </c>
-      <c r="I29" s="36">
-        <f>I7+I8+I9+I10+I11+I12+I13+I14+I15+I16+I17+I18</f>
-      </c>
-      <c r="J29" s="36">
-        <f>J7+J8+J9+J10+J11+J12+J13+J14+J15+J16+J17+J18</f>
-      </c>
-      <c r="K29" s="36">
-        <f>K7+K8+K9+K10+K11+K12+K13+K14+K15+K16+K17+K18</f>
-      </c>
-      <c r="L29" s="36">
-        <f>L7+L8+L9+L10+L11+L12+L13+L14+L15+L16+L17+L18</f>
-      </c>
-      <c r="M29" s="36">
-        <f>M7+M8+M9+M10+M11+M12+M13+M14+M15+M16+M17+M18</f>
-      </c>
-      <c r="N29" s="36">
-        <f>N7+N8+N9+N10+N11+N12+N13+N14+N15+N16+N17+N18</f>
-      </c>
-      <c r="O29" s="36">
-        <f>O7+O8+O9+O10+O11+O12+O13+O14+O15+O16+O17+O18</f>
-      </c>
-      <c r="P29" s="36">
+      <c r="D29" s="37">
+        <f>D7+D8+D9*Configuración!$C$22+D10*Configuración!$C$23+D11*Configuración!$C$24+D12*Configuración!$C$25+D13*Configuración!$C$26+D14*Configuración!$C$27+D15*Configuración!$C$28+D16*Configuración!$C$31+D17*Configuración!$C$29+D18*Configuración!$C$30</f>
+      </c>
+      <c r="E29" s="37">
+        <f>E7+E8+E9*Configuración!$C$22+E10*Configuración!$C$23+E11*Configuración!$C$24+E12*Configuración!$C$25+E13*Configuración!$C$26+E14*Configuración!$C$27+E15*Configuración!$C$28+E16*Configuración!$C$31+E17*Configuración!$C$29+E18*Configuración!$C$30</f>
+      </c>
+      <c r="F29" s="37">
+        <f>F7+F8+F9*Configuración!$C$22+F10*Configuración!$C$23+F11*Configuración!$C$24+F12*Configuración!$C$25+F13*Configuración!$C$26+F14*Configuración!$C$27+F15*Configuración!$C$28+F16*Configuración!$C$31+F17*Configuración!$C$29+F18*Configuración!$C$30</f>
+      </c>
+      <c r="G29" s="37">
+        <f>G7+G8+G9*Configuración!$C$22+G10*Configuración!$C$23+G11*Configuración!$C$24+G12*Configuración!$C$25+G13*Configuración!$C$26+G14*Configuración!$C$27+G15*Configuración!$C$28+G16*Configuración!$C$31+G17*Configuración!$C$29+G18*Configuración!$C$30</f>
+      </c>
+      <c r="H29" s="37">
+        <f>H7+H8+H9*Configuración!$C$22+H10*Configuración!$C$23+H11*Configuración!$C$24+H12*Configuración!$C$25+H13*Configuración!$C$26+H14*Configuración!$C$27+H15*Configuración!$C$28+H16*Configuración!$C$31+H17*Configuración!$C$29+H18*Configuración!$C$30</f>
+      </c>
+      <c r="I29" s="37">
+        <f>I7+I8+I9*Configuración!$C$22+I10*Configuración!$C$23+I11*Configuración!$C$24+I12*Configuración!$C$25+I13*Configuración!$C$26+I14*Configuración!$C$27+I15*Configuración!$C$28+I16*Configuración!$C$31+I17*Configuración!$C$29+I18*Configuración!$C$30</f>
+      </c>
+      <c r="J29" s="37">
+        <f>J7+J8+J9*Configuración!$C$22+J10*Configuración!$C$23+J11*Configuración!$C$24+J12*Configuración!$C$25+J13*Configuración!$C$26+J14*Configuración!$C$27+J15*Configuración!$C$28+J16*Configuración!$C$31+J17*Configuración!$C$29+J18*Configuración!$C$30</f>
+      </c>
+      <c r="K29" s="37">
+        <f>K7+K8+K9*Configuración!$C$22+K10*Configuración!$C$23+K11*Configuración!$C$24+K12*Configuración!$C$25+K13*Configuración!$C$26+K14*Configuración!$C$27+K15*Configuración!$C$28+K16*Configuración!$C$31+K17*Configuración!$C$29+K18*Configuración!$C$30</f>
+      </c>
+      <c r="L29" s="37">
+        <f>L7+L8+L9*Configuración!$C$22+L10*Configuración!$C$23+L11*Configuración!$C$24+L12*Configuración!$C$25+L13*Configuración!$C$26+L14*Configuración!$C$27+L15*Configuración!$C$28+L16*Configuración!$C$31+L17*Configuración!$C$29+L18*Configuración!$C$30</f>
+      </c>
+      <c r="M29" s="37">
+        <f>M7+M8+M9*Configuración!$C$22+M10*Configuración!$C$23+M11*Configuración!$C$24+M12*Configuración!$C$25+M13*Configuración!$C$26+M14*Configuración!$C$27+M15*Configuración!$C$28+M16*Configuración!$C$31+M17*Configuración!$C$29+M18*Configuración!$C$30</f>
+      </c>
+      <c r="N29" s="37">
+        <f>N7+N8+N9*Configuración!$C$22+N10*Configuración!$C$23+N11*Configuración!$C$24+N12*Configuración!$C$25+N13*Configuración!$C$26+N14*Configuración!$C$27+N15*Configuración!$C$28+N16*Configuración!$C$31+N17*Configuración!$C$29+N18*Configuración!$C$30</f>
+      </c>
+      <c r="O29" s="37">
+        <f>O7+O8+O9*Configuración!$C$22+O10*Configuración!$C$23+O11*Configuración!$C$24+O12*Configuración!$C$25+O13*Configuración!$C$26+O14*Configuración!$C$27+O15*Configuración!$C$28+O16*Configuración!$C$31+O17*Configuración!$C$29+O18*Configuración!$C$30</f>
+      </c>
+      <c r="P29" s="37">
         <f>SUM(D29:O29)</f>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B30" s="37" t="s">
+      <c r="B30" s="38" t="s">
         <v>93</v>
       </c>
       <c r="C30" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="D30" s="38">
-        <f>D17+D18</f>
-      </c>
-      <c r="E30" s="38">
-        <f>E17+E18</f>
-      </c>
-      <c r="F30" s="38">
-        <f>F17+F18</f>
-      </c>
-      <c r="G30" s="38">
-        <f>G17+G18</f>
-      </c>
-      <c r="H30" s="38">
-        <f>H17+H18</f>
-      </c>
-      <c r="I30" s="38">
-        <f>I17+I18</f>
-      </c>
-      <c r="J30" s="38">
-        <f>J17+J18</f>
-      </c>
-      <c r="K30" s="38">
-        <f>K17+K18</f>
-      </c>
-      <c r="L30" s="38">
-        <f>L17+L18</f>
-      </c>
-      <c r="M30" s="38">
-        <f>M17+M18</f>
-      </c>
-      <c r="N30" s="38">
-        <f>N17+N18</f>
-      </c>
-      <c r="O30" s="38">
-        <f>O17+O18</f>
+      <c r="D30" s="39">
+        <f>D17*Configuración!$C$29+D18*Configuración!$C$30</f>
+      </c>
+      <c r="E30" s="39">
+        <f>E17*Configuración!$C$29+E18*Configuración!$C$30</f>
+      </c>
+      <c r="F30" s="39">
+        <f>F17*Configuración!$C$29+F18*Configuración!$C$30</f>
+      </c>
+      <c r="G30" s="39">
+        <f>G17*Configuración!$C$29+G18*Configuración!$C$30</f>
+      </c>
+      <c r="H30" s="39">
+        <f>H17*Configuración!$C$29+H18*Configuración!$C$30</f>
+      </c>
+      <c r="I30" s="39">
+        <f>I17*Configuración!$C$29+I18*Configuración!$C$30</f>
+      </c>
+      <c r="J30" s="39">
+        <f>J17*Configuración!$C$29+J18*Configuración!$C$30</f>
+      </c>
+      <c r="K30" s="39">
+        <f>K17*Configuración!$C$29+K18*Configuración!$C$30</f>
+      </c>
+      <c r="L30" s="39">
+        <f>L17*Configuración!$C$29+L18*Configuración!$C$30</f>
+      </c>
+      <c r="M30" s="39">
+        <f>M17*Configuración!$C$29+M18*Configuración!$C$30</f>
+      </c>
+      <c r="N30" s="39">
+        <f>N17*Configuración!$C$29+N18*Configuración!$C$30</f>
+      </c>
+      <c r="O30" s="39">
+        <f>O17*Configuración!$C$29+O18*Configuración!$C$30</f>
       </c>
       <c r="P30" s="25">
         <f>SUM(D30:O30)</f>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B31" s="29" t="s">
+      <c r="B31" s="30" t="s">
         <v>95</v>
       </c>
-      <c r="C31" s="30" t="s">
+      <c r="C31" s="31" t="s">
         <v>84</v>
       </c>
-      <c r="D31" s="39">
-        <f>D21+D22+D23</f>
-      </c>
-      <c r="E31" s="39">
-        <f>E21+E22+E23</f>
-      </c>
-      <c r="F31" s="39">
-        <f>F21+F22+F23</f>
-      </c>
-      <c r="G31" s="39">
-        <f>G21+G22+G23</f>
-      </c>
-      <c r="H31" s="39">
-        <f>H21+H22+H23</f>
-      </c>
-      <c r="I31" s="39">
-        <f>I21+I22+I23</f>
-      </c>
-      <c r="J31" s="39">
-        <f>J21+J22+J23</f>
-      </c>
-      <c r="K31" s="39">
-        <f>K21+K22+K23</f>
-      </c>
-      <c r="L31" s="39">
-        <f>L21+L22+L23</f>
-      </c>
-      <c r="M31" s="39">
-        <f>M21+M22+M23</f>
-      </c>
-      <c r="N31" s="39">
-        <f>N21+N22+N23</f>
-      </c>
-      <c r="O31" s="39">
-        <f>O21+O22+O23</f>
+      <c r="D31" s="40">
+        <f>D21+D22+D23*Configuración!$C$32</f>
+      </c>
+      <c r="E31" s="40">
+        <f>E21+E22+E23*Configuración!$C$32</f>
+      </c>
+      <c r="F31" s="40">
+        <f>F21+F22+F23*Configuración!$C$32</f>
+      </c>
+      <c r="G31" s="40">
+        <f>G21+G22+G23*Configuración!$C$32</f>
+      </c>
+      <c r="H31" s="40">
+        <f>H21+H22+H23*Configuración!$C$32</f>
+      </c>
+      <c r="I31" s="40">
+        <f>I21+I22+I23*Configuración!$C$32</f>
+      </c>
+      <c r="J31" s="40">
+        <f>J21+J22+J23*Configuración!$C$32</f>
+      </c>
+      <c r="K31" s="40">
+        <f>K21+K22+K23*Configuración!$C$32</f>
+      </c>
+      <c r="L31" s="40">
+        <f>L21+L22+L23*Configuración!$C$32</f>
+      </c>
+      <c r="M31" s="40">
+        <f>M21+M22+M23*Configuración!$C$32</f>
+      </c>
+      <c r="N31" s="40">
+        <f>N21+N22+N23*Configuración!$C$32</f>
+      </c>
+      <c r="O31" s="40">
+        <f>O21+O22+O23*Configuración!$C$32</f>
       </c>
       <c r="P31" s="25">
         <f>SUM(D31:O31)</f>
@@ -2942,63 +2942,63 @@
       <c r="P32" s="20"/>
     </row>
     <row r="33" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A33" s="40" t="s">
+      <c r="A33" s="41" t="s">
         <v>96</v>
       </c>
-      <c r="B33" s="40"/>
-      <c r="C33" s="40"/>
-      <c r="D33" s="40"/>
-      <c r="E33" s="40"/>
-      <c r="F33" s="40"/>
-      <c r="G33" s="40"/>
-      <c r="H33" s="40"/>
-      <c r="I33" s="40"/>
-      <c r="J33" s="40"/>
-      <c r="K33" s="40"/>
-      <c r="L33" s="40"/>
-      <c r="M33" s="40"/>
-      <c r="N33" s="40"/>
-      <c r="O33" s="40"/>
-      <c r="P33" s="40"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="41"/>
+      <c r="H33" s="41"/>
+      <c r="I33" s="41"/>
+      <c r="J33" s="41"/>
+      <c r="K33" s="41"/>
+      <c r="L33" s="41"/>
+      <c r="M33" s="41"/>
+      <c r="N33" s="41"/>
+      <c r="O33" s="41"/>
+      <c r="P33" s="41"/>
     </row>
     <row r="34" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B34" s="41" t="s">
+      <c r="B34" s="42" t="s">
         <v>97</v>
       </c>
-      <c r="D34" s="42">
+      <c r="D34" s="43">
         <f>D29-D30+Configuración!$C$7</f>
       </c>
-      <c r="E34" s="42">
+      <c r="E34" s="43">
         <f>E29-E30+Configuración!$C$7</f>
       </c>
-      <c r="F34" s="42">
+      <c r="F34" s="43">
         <f>F29-F30+Configuración!$C$7</f>
       </c>
-      <c r="G34" s="42">
+      <c r="G34" s="43">
         <f>G29-G30+Configuración!$C$7</f>
       </c>
-      <c r="H34" s="42">
+      <c r="H34" s="43">
         <f>H29-H30+Configuración!$C$7</f>
       </c>
-      <c r="I34" s="42">
+      <c r="I34" s="43">
         <f>I29-I30+Configuración!$C$7</f>
       </c>
-      <c r="J34" s="42">
+      <c r="J34" s="43">
         <f>J29-J30+Configuración!$C$7</f>
       </c>
-      <c r="K34" s="42">
+      <c r="K34" s="43">
         <f>K29-K30+Configuración!$C$7</f>
       </c>
-      <c r="L34" s="42">
+      <c r="L34" s="43">
         <f>L29-L30+Configuración!$C$7</f>
       </c>
-      <c r="M34" s="42">
+      <c r="M34" s="43">
         <f>M29-M30+Configuración!$C$7</f>
       </c>
-      <c r="N34" s="42">
+      <c r="N34" s="43">
         <f>N29-N30+Configuración!$C$7</f>
       </c>
-      <c r="O34" s="42">
+      <c r="O34" s="43">
         <f>O29-O30+Configuración!$C$7</f>
       </c>
       <c r="P34" s="25">
@@ -3006,43 +3006,43 @@
       </c>
     </row>
     <row r="35" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B35" s="41" t="s">
+      <c r="B35" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="D35" s="42">
+      <c r="D35" s="43">
         <f>D34+D30</f>
       </c>
-      <c r="E35" s="42">
+      <c r="E35" s="43">
         <f>E34+E30</f>
       </c>
-      <c r="F35" s="42">
+      <c r="F35" s="43">
         <f>F34+F30</f>
       </c>
-      <c r="G35" s="42">
+      <c r="G35" s="43">
         <f>G34+G30</f>
       </c>
-      <c r="H35" s="42">
+      <c r="H35" s="43">
         <f>H34+H30</f>
       </c>
-      <c r="I35" s="42">
+      <c r="I35" s="43">
         <f>I34+I30</f>
       </c>
-      <c r="J35" s="42">
+      <c r="J35" s="43">
         <f>J34+J30</f>
       </c>
-      <c r="K35" s="42">
+      <c r="K35" s="43">
         <f>K34+K30</f>
       </c>
-      <c r="L35" s="42">
+      <c r="L35" s="43">
         <f>L34+L30</f>
       </c>
-      <c r="M35" s="42">
+      <c r="M35" s="43">
         <f>M34+M30</f>
       </c>
-      <c r="N35" s="42">
+      <c r="N35" s="43">
         <f>N34+N30</f>
       </c>
-      <c r="O35" s="42">
+      <c r="O35" s="43">
         <f>O34+O30</f>
       </c>
       <c r="P35" s="25">
@@ -3050,46 +3050,46 @@
       </c>
     </row>
     <row r="36" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B36" s="43" t="s">
+      <c r="B36" s="44" t="s">
         <v>98</v>
       </c>
-      <c r="C36" s="44" t="s">
+      <c r="C36" s="45" t="s">
         <v>99</v>
       </c>
-      <c r="D36" s="45">
+      <c r="D36" s="46">
         <f>D34*Configuración!$C$12</f>
       </c>
-      <c r="E36" s="45">
+      <c r="E36" s="46">
         <f>E34*Configuración!$C$12</f>
       </c>
-      <c r="F36" s="45">
+      <c r="F36" s="46">
         <f>F34*Configuración!$C$12</f>
       </c>
-      <c r="G36" s="45">
+      <c r="G36" s="46">
         <f>G34*Configuración!$C$12</f>
       </c>
-      <c r="H36" s="45">
+      <c r="H36" s="46">
         <f>H34*Configuración!$C$12</f>
       </c>
-      <c r="I36" s="45">
+      <c r="I36" s="46">
         <f>I34*Configuración!$C$12</f>
       </c>
-      <c r="J36" s="45">
+      <c r="J36" s="46">
         <f>J34*Configuración!$C$12</f>
       </c>
-      <c r="K36" s="45">
+      <c r="K36" s="46">
         <f>K34*Configuración!$C$12</f>
       </c>
-      <c r="L36" s="45">
+      <c r="L36" s="46">
         <f>L34*Configuración!$C$12</f>
       </c>
-      <c r="M36" s="45">
+      <c r="M36" s="46">
         <f>M34*Configuración!$C$12</f>
       </c>
-      <c r="N36" s="45">
+      <c r="N36" s="46">
         <f>N34*Configuración!$C$12</f>
       </c>
-      <c r="O36" s="45">
+      <c r="O36" s="46">
         <f>O34*Configuración!$C$12</f>
       </c>
       <c r="P36" s="25">
@@ -3097,46 +3097,46 @@
       </c>
     </row>
     <row r="37" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B37" s="43" t="s">
+      <c r="B37" s="44" t="s">
         <v>100</v>
       </c>
-      <c r="C37" s="44" t="s">
+      <c r="C37" s="45" t="s">
         <v>101</v>
       </c>
-      <c r="D37" s="45">
+      <c r="D37" s="46">
         <f>D35*Configuración!$C$13</f>
       </c>
-      <c r="E37" s="45">
+      <c r="E37" s="46">
         <f>E35*Configuración!$C$13</f>
       </c>
-      <c r="F37" s="45">
+      <c r="F37" s="46">
         <f>F35*Configuración!$C$13</f>
       </c>
-      <c r="G37" s="45">
+      <c r="G37" s="46">
         <f>G35*Configuración!$C$13</f>
       </c>
-      <c r="H37" s="45">
+      <c r="H37" s="46">
         <f>H35*Configuración!$C$13</f>
       </c>
-      <c r="I37" s="45">
+      <c r="I37" s="46">
         <f>I35*Configuración!$C$13</f>
       </c>
-      <c r="J37" s="45">
+      <c r="J37" s="46">
         <f>J35*Configuración!$C$13</f>
       </c>
-      <c r="K37" s="45">
+      <c r="K37" s="46">
         <f>K35*Configuración!$C$13</f>
       </c>
-      <c r="L37" s="45">
+      <c r="L37" s="46">
         <f>L35*Configuración!$C$13</f>
       </c>
-      <c r="M37" s="45">
+      <c r="M37" s="46">
         <f>M35*Configuración!$C$13</f>
       </c>
-      <c r="N37" s="45">
+      <c r="N37" s="46">
         <f>N35*Configuración!$C$13</f>
       </c>
-      <c r="O37" s="45">
+      <c r="O37" s="46">
         <f>O35*Configuración!$C$13</f>
       </c>
       <c r="P37" s="25">
@@ -3144,46 +3144,46 @@
       </c>
     </row>
     <row r="38" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B38" s="43" t="s">
+      <c r="B38" s="44" t="s">
         <v>102</v>
       </c>
-      <c r="C38" s="44" t="s">
+      <c r="C38" s="45" t="s">
         <v>99</v>
       </c>
-      <c r="D38" s="45">
+      <c r="D38" s="46">
         <f>D30*Configuración!$C$14</f>
       </c>
-      <c r="E38" s="45">
+      <c r="E38" s="46">
         <f>E30*Configuración!$C$14</f>
       </c>
-      <c r="F38" s="45">
+      <c r="F38" s="46">
         <f>F30*Configuración!$C$14</f>
       </c>
-      <c r="G38" s="45">
+      <c r="G38" s="46">
         <f>G30*Configuración!$C$14</f>
       </c>
-      <c r="H38" s="45">
+      <c r="H38" s="46">
         <f>H30*Configuración!$C$14</f>
       </c>
-      <c r="I38" s="45">
+      <c r="I38" s="46">
         <f>I30*Configuración!$C$14</f>
       </c>
-      <c r="J38" s="45">
+      <c r="J38" s="46">
         <f>J30*Configuración!$C$14</f>
       </c>
-      <c r="K38" s="45">
+      <c r="K38" s="46">
         <f>K30*Configuración!$C$14</f>
       </c>
-      <c r="L38" s="45">
+      <c r="L38" s="46">
         <f>L30*Configuración!$C$14</f>
       </c>
-      <c r="M38" s="45">
+      <c r="M38" s="46">
         <f>M30*Configuración!$C$14</f>
       </c>
-      <c r="N38" s="45">
+      <c r="N38" s="46">
         <f>N30*Configuración!$C$14</f>
       </c>
-      <c r="O38" s="45">
+      <c r="O38" s="46">
         <f>O30*Configuración!$C$14</f>
       </c>
       <c r="P38" s="25">
@@ -3191,46 +3191,46 @@
       </c>
     </row>
     <row r="39" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B39" s="43" t="s">
+      <c r="B39" s="44" t="s">
         <v>103</v>
       </c>
-      <c r="C39" s="44" t="s">
+      <c r="C39" s="45" t="s">
         <v>104</v>
       </c>
-      <c r="D39" s="45">
+      <c r="D39" s="46">
         <f>D35*Configuración!$C$15</f>
       </c>
-      <c r="E39" s="45">
+      <c r="E39" s="46">
         <f>E35*Configuración!$C$15</f>
       </c>
-      <c r="F39" s="45">
+      <c r="F39" s="46">
         <f>F35*Configuración!$C$15</f>
       </c>
-      <c r="G39" s="45">
+      <c r="G39" s="46">
         <f>G35*Configuración!$C$15</f>
       </c>
-      <c r="H39" s="45">
+      <c r="H39" s="46">
         <f>H35*Configuración!$C$15</f>
       </c>
-      <c r="I39" s="45">
+      <c r="I39" s="46">
         <f>I35*Configuración!$C$15</f>
       </c>
-      <c r="J39" s="45">
+      <c r="J39" s="46">
         <f>J35*Configuración!$C$15</f>
       </c>
-      <c r="K39" s="45">
+      <c r="K39" s="46">
         <f>K35*Configuración!$C$15</f>
       </c>
-      <c r="L39" s="45">
+      <c r="L39" s="46">
         <f>L35*Configuración!$C$15</f>
       </c>
-      <c r="M39" s="45">
+      <c r="M39" s="46">
         <f>M35*Configuración!$C$15</f>
       </c>
-      <c r="N39" s="45">
+      <c r="N39" s="46">
         <f>N35*Configuración!$C$15</f>
       </c>
-      <c r="O39" s="45">
+      <c r="O39" s="46">
         <f>O35*Configuración!$C$15</f>
       </c>
       <c r="P39" s="25">
@@ -3238,46 +3238,46 @@
       </c>
     </row>
     <row r="40" ht="22" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B40" s="46" t="s">
+      <c r="B40" s="47" t="s">
         <v>105</v>
       </c>
-      <c r="D40" s="47">
+      <c r="D40" s="48">
         <f>D36+D37+D38+D39</f>
       </c>
-      <c r="E40" s="47">
+      <c r="E40" s="48">
         <f>E36+E37+E38+E39</f>
       </c>
-      <c r="F40" s="47">
+      <c r="F40" s="48">
         <f>F36+F37+F38+F39</f>
       </c>
-      <c r="G40" s="47">
+      <c r="G40" s="48">
         <f>G36+G37+G38+G39</f>
       </c>
-      <c r="H40" s="47">
+      <c r="H40" s="48">
         <f>H36+H37+H38+H39</f>
       </c>
-      <c r="I40" s="47">
+      <c r="I40" s="48">
         <f>I36+I37+I38+I39</f>
       </c>
-      <c r="J40" s="47">
+      <c r="J40" s="48">
         <f>J36+J37+J38+J39</f>
       </c>
-      <c r="K40" s="47">
+      <c r="K40" s="48">
         <f>K36+K37+K38+K39</f>
       </c>
-      <c r="L40" s="47">
+      <c r="L40" s="48">
         <f>L36+L37+L38+L39</f>
       </c>
-      <c r="M40" s="47">
+      <c r="M40" s="48">
         <f>M36+M37+M38+M39</f>
       </c>
-      <c r="N40" s="47">
+      <c r="N40" s="48">
         <f>N36+N37+N38+N39</f>
       </c>
-      <c r="O40" s="47">
+      <c r="O40" s="48">
         <f>O36+O37+O38+O39</f>
       </c>
-      <c r="P40" s="47">
+      <c r="P40" s="48">
         <f>SUM(D40:O40)</f>
       </c>
     </row>
@@ -3300,63 +3300,63 @@
       <c r="P41" s="20"/>
     </row>
     <row r="42" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A42" s="31" t="s">
+      <c r="A42" s="32" t="s">
         <v>106</v>
       </c>
-      <c r="B42" s="31"/>
-      <c r="C42" s="31"/>
-      <c r="D42" s="31"/>
-      <c r="E42" s="31"/>
-      <c r="F42" s="31"/>
-      <c r="G42" s="31"/>
-      <c r="H42" s="31"/>
-      <c r="I42" s="31"/>
-      <c r="J42" s="31"/>
-      <c r="K42" s="31"/>
-      <c r="L42" s="31"/>
-      <c r="M42" s="31"/>
-      <c r="N42" s="31"/>
-      <c r="O42" s="31"/>
-      <c r="P42" s="31"/>
+      <c r="B42" s="32"/>
+      <c r="C42" s="32"/>
+      <c r="D42" s="32"/>
+      <c r="E42" s="32"/>
+      <c r="F42" s="32"/>
+      <c r="G42" s="32"/>
+      <c r="H42" s="32"/>
+      <c r="I42" s="32"/>
+      <c r="J42" s="32"/>
+      <c r="K42" s="32"/>
+      <c r="L42" s="32"/>
+      <c r="M42" s="32"/>
+      <c r="N42" s="32"/>
+      <c r="O42" s="32"/>
+      <c r="P42" s="32"/>
     </row>
     <row r="43" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B43" s="32" t="s">
+      <c r="B43" s="33" t="s">
         <v>107</v>
       </c>
-      <c r="D43" s="48">
+      <c r="D43" s="49">
         <f>D26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="E43" s="48">
+      <c r="E43" s="49">
         <f>E26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="F43" s="48">
+      <c r="F43" s="49">
         <f>F26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="G43" s="48">
+      <c r="G43" s="49">
         <f>G26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="H43" s="48">
+      <c r="H43" s="49">
         <f>H26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="I43" s="48">
+      <c r="I43" s="49">
         <f>I26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="J43" s="48">
+      <c r="J43" s="49">
         <f>J26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="K43" s="48">
+      <c r="K43" s="49">
         <f>K26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="L43" s="48">
+      <c r="L43" s="49">
         <f>L26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="M43" s="48">
+      <c r="M43" s="49">
         <f>M26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="N43" s="48">
+      <c r="N43" s="49">
         <f>N26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="O43" s="48">
+      <c r="O43" s="49">
         <f>O26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
       <c r="P43" s="25">
@@ -3364,43 +3364,43 @@
       </c>
     </row>
     <row r="44" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B44" s="32" t="s">
+      <c r="B44" s="33" t="s">
         <v>108</v>
       </c>
-      <c r="D44" s="48">
+      <c r="D44" s="49">
         <f>D26*D4</f>
       </c>
-      <c r="E44" s="48">
+      <c r="E44" s="49">
         <f>E26*E4</f>
       </c>
-      <c r="F44" s="48">
+      <c r="F44" s="49">
         <f>F26*F4</f>
       </c>
-      <c r="G44" s="48">
+      <c r="G44" s="49">
         <f>G26*G4</f>
       </c>
-      <c r="H44" s="48">
+      <c r="H44" s="49">
         <f>H26*H4</f>
       </c>
-      <c r="I44" s="48">
+      <c r="I44" s="49">
         <f>I26*I4</f>
       </c>
-      <c r="J44" s="48">
+      <c r="J44" s="49">
         <f>J26*J4</f>
       </c>
-      <c r="K44" s="48">
+      <c r="K44" s="49">
         <f>K26*K4</f>
       </c>
-      <c r="L44" s="48">
+      <c r="L44" s="49">
         <f>L26*L4</f>
       </c>
-      <c r="M44" s="48">
+      <c r="M44" s="49">
         <f>M26*M4</f>
       </c>
-      <c r="N44" s="48">
+      <c r="N44" s="49">
         <f>N26*N4</f>
       </c>
-      <c r="O44" s="48">
+      <c r="O44" s="49">
         <f>O26*O4</f>
       </c>
       <c r="P44" s="25">
@@ -3408,46 +3408,46 @@
       </c>
     </row>
     <row r="45" ht="20" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B45" s="49" t="s">
+      <c r="B45" s="50" t="s">
         <v>109</v>
       </c>
-      <c r="D45" s="50">
+      <c r="D45" s="51">
         <f>D26-D43-D44</f>
       </c>
-      <c r="E45" s="50">
+      <c r="E45" s="51">
         <f>E26-E43-E44</f>
       </c>
-      <c r="F45" s="50">
+      <c r="F45" s="51">
         <f>F26-F43-F44</f>
       </c>
-      <c r="G45" s="50">
+      <c r="G45" s="51">
         <f>G26-G43-G44</f>
       </c>
-      <c r="H45" s="50">
+      <c r="H45" s="51">
         <f>H26-H43-H44</f>
       </c>
-      <c r="I45" s="50">
+      <c r="I45" s="51">
         <f>I26-I43-I44</f>
       </c>
-      <c r="J45" s="50">
+      <c r="J45" s="51">
         <f>J26-J43-J44</f>
       </c>
-      <c r="K45" s="50">
+      <c r="K45" s="51">
         <f>K26-K43-K44</f>
       </c>
-      <c r="L45" s="50">
+      <c r="L45" s="51">
         <f>L26-L43-L44</f>
       </c>
-      <c r="M45" s="50">
+      <c r="M45" s="51">
         <f>M26-M43-M44</f>
       </c>
-      <c r="N45" s="50">
+      <c r="N45" s="51">
         <f>N26-N43-N44</f>
       </c>
-      <c r="O45" s="50">
+      <c r="O45" s="51">
         <f>O26-O43-O44</f>
       </c>
-      <c r="P45" s="50">
+      <c r="P45" s="51">
         <f>SUM(D45:O45)</f>
       </c>
     </row>
@@ -3470,43 +3470,43 @@
       <c r="P46" s="20"/>
     </row>
     <row r="47" ht="20" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B47" s="43" t="s">
+      <c r="B47" s="44" t="s">
         <v>110</v>
       </c>
-      <c r="D47" s="45">
+      <c r="D47" s="46">
         <f>D29*D4</f>
       </c>
-      <c r="E47" s="45">
+      <c r="E47" s="46">
         <f>E29*E4</f>
       </c>
-      <c r="F47" s="45">
+      <c r="F47" s="46">
         <f>F29*F4</f>
       </c>
-      <c r="G47" s="45">
+      <c r="G47" s="46">
         <f>G29*G4</f>
       </c>
-      <c r="H47" s="45">
+      <c r="H47" s="46">
         <f>H29*H4</f>
       </c>
-      <c r="I47" s="45">
+      <c r="I47" s="46">
         <f>I29*I4</f>
       </c>
-      <c r="J47" s="45">
+      <c r="J47" s="46">
         <f>J29*J4</f>
       </c>
-      <c r="K47" s="45">
+      <c r="K47" s="46">
         <f>K29*K4</f>
       </c>
-      <c r="L47" s="45">
+      <c r="L47" s="46">
         <f>L29*L4</f>
       </c>
-      <c r="M47" s="45">
+      <c r="M47" s="46">
         <f>M29*M4</f>
       </c>
-      <c r="N47" s="45">
+      <c r="N47" s="46">
         <f>N29*N4</f>
       </c>
-      <c r="O47" s="45">
+      <c r="O47" s="46">
         <f>O29*O4</f>
       </c>
       <c r="P47" s="25">
@@ -3514,96 +3514,96 @@
       </c>
     </row>
     <row r="48" ht="26" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B48" s="51" t="s">
+      <c r="B48" s="52" t="s">
         <v>111</v>
       </c>
-      <c r="C48" s="52" t="s">
+      <c r="C48" s="53" t="s">
         <v>112</v>
       </c>
-      <c r="D48" s="53">
+      <c r="D48" s="54">
         <f>D29+D31-D40-D47</f>
       </c>
-      <c r="E48" s="53">
+      <c r="E48" s="54">
         <f>E29+E31-E40-E47</f>
       </c>
-      <c r="F48" s="53">
+      <c r="F48" s="54">
         <f>F29+F31-F40-F47</f>
       </c>
-      <c r="G48" s="53">
+      <c r="G48" s="54">
         <f>G29+G31-G40-G47</f>
       </c>
-      <c r="H48" s="53">
+      <c r="H48" s="54">
         <f>H29+H31-H40-H47</f>
       </c>
-      <c r="I48" s="53">
+      <c r="I48" s="54">
         <f>I29+I31-I40-I47</f>
       </c>
-      <c r="J48" s="53">
+      <c r="J48" s="54">
         <f>J29+J31-J40-J47</f>
       </c>
-      <c r="K48" s="53">
+      <c r="K48" s="54">
         <f>K29+K31-K40-K47</f>
       </c>
-      <c r="L48" s="53">
+      <c r="L48" s="54">
         <f>L29+L31-L40-L47</f>
       </c>
-      <c r="M48" s="53">
+      <c r="M48" s="54">
         <f>M29+M31-M40-M47</f>
       </c>
-      <c r="N48" s="53">
+      <c r="N48" s="54">
         <f>N29+N31-N40-N47</f>
       </c>
-      <c r="O48" s="53">
+      <c r="O48" s="54">
         <f>O29+O31-O40-O47</f>
       </c>
-      <c r="P48" s="53">
+      <c r="P48" s="54">
         <f>SUM(D48:O48)</f>
       </c>
     </row>
     <row r="49" ht="28" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B49" s="51" t="s">
+      <c r="B49" s="52" t="s">
         <v>113</v>
       </c>
-      <c r="C49" s="52" t="s">
+      <c r="C49" s="53" t="s">
         <v>114</v>
       </c>
-      <c r="D49" s="53">
+      <c r="D49" s="54">
         <f>D48+D45</f>
       </c>
-      <c r="E49" s="53">
+      <c r="E49" s="54">
         <f>E48+E45</f>
       </c>
-      <c r="F49" s="53">
+      <c r="F49" s="54">
         <f>F48+F45</f>
       </c>
-      <c r="G49" s="53">
+      <c r="G49" s="54">
         <f>G48+G45</f>
       </c>
-      <c r="H49" s="53">
+      <c r="H49" s="54">
         <f>H48+H45</f>
       </c>
-      <c r="I49" s="53">
+      <c r="I49" s="54">
         <f>I48+I45</f>
       </c>
-      <c r="J49" s="53">
+      <c r="J49" s="54">
         <f>J48+J45</f>
       </c>
-      <c r="K49" s="53">
+      <c r="K49" s="54">
         <f>K48+K45</f>
       </c>
-      <c r="L49" s="53">
+      <c r="L49" s="54">
         <f>L48+L45</f>
       </c>
-      <c r="M49" s="53">
+      <c r="M49" s="54">
         <f>M48+M45</f>
       </c>
-      <c r="N49" s="53">
+      <c r="N49" s="54">
         <f>N48+N45</f>
       </c>
-      <c r="O49" s="53">
+      <c r="O49" s="54">
         <f>O48+O45</f>
       </c>
-      <c r="P49" s="53">
+      <c r="P49" s="54">
         <f>SUM(D49:O49)</f>
       </c>
     </row>
@@ -3626,77 +3626,77 @@
       <c r="P50" s="2"/>
     </row>
     <row r="51" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A51" s="54" t="s">
+      <c r="A51" s="55" t="s">
         <v>115</v>
       </c>
-      <c r="B51" s="54"/>
-      <c r="C51" s="54"/>
-      <c r="D51" s="54"/>
-      <c r="E51" s="54"/>
-      <c r="F51" s="54"/>
-      <c r="G51" s="54"/>
-      <c r="H51" s="54"/>
-      <c r="I51" s="54"/>
-      <c r="J51" s="54"/>
-      <c r="K51" s="54"/>
-      <c r="L51" s="54"/>
-      <c r="M51" s="54"/>
-      <c r="N51" s="54"/>
-      <c r="O51" s="54"/>
-      <c r="P51" s="54"/>
+      <c r="B51" s="55"/>
+      <c r="C51" s="55"/>
+      <c r="D51" s="55"/>
+      <c r="E51" s="55"/>
+      <c r="F51" s="55"/>
+      <c r="G51" s="55"/>
+      <c r="H51" s="55"/>
+      <c r="I51" s="55"/>
+      <c r="J51" s="55"/>
+      <c r="K51" s="55"/>
+      <c r="L51" s="55"/>
+      <c r="M51" s="55"/>
+      <c r="N51" s="55"/>
+      <c r="O51" s="55"/>
+      <c r="P51" s="55"/>
     </row>
     <row r="52" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B52" s="55" t="s">
+      <c r="B52" s="56" t="s">
         <v>116</v>
       </c>
-      <c r="C52" s="56" t="s">
+      <c r="C52" s="57" t="s">
         <v>117</v>
       </c>
-      <c r="D52" s="57">
-        <v>0</v>
-      </c>
-      <c r="E52" s="57">
-        <v>0</v>
-      </c>
-      <c r="F52" s="57">
-        <v>0</v>
-      </c>
-      <c r="G52" s="57">
-        <v>0</v>
-      </c>
-      <c r="H52" s="57">
-        <v>0</v>
-      </c>
-      <c r="I52" s="57">
-        <v>0</v>
-      </c>
-      <c r="J52" s="57">
-        <v>0</v>
-      </c>
-      <c r="K52" s="57">
-        <v>0</v>
-      </c>
-      <c r="L52" s="57">
-        <v>0</v>
-      </c>
-      <c r="M52" s="57">
-        <v>0</v>
-      </c>
-      <c r="N52" s="57">
-        <v>0</v>
-      </c>
-      <c r="O52" s="57">
-        <v>0</v>
-      </c>
-      <c r="P52" s="58">
+      <c r="D52" s="58">
+        <f>D16</f>
+      </c>
+      <c r="E52" s="58">
+        <f>E16</f>
+      </c>
+      <c r="F52" s="58">
+        <f>F16</f>
+      </c>
+      <c r="G52" s="58">
+        <f>G16</f>
+      </c>
+      <c r="H52" s="58">
+        <f>H16</f>
+      </c>
+      <c r="I52" s="58">
+        <f>I16</f>
+      </c>
+      <c r="J52" s="58">
+        <f>J16</f>
+      </c>
+      <c r="K52" s="58">
+        <f>K16</f>
+      </c>
+      <c r="L52" s="58">
+        <f>L16</f>
+      </c>
+      <c r="M52" s="58">
+        <f>M16</f>
+      </c>
+      <c r="N52" s="58">
+        <f>N16</f>
+      </c>
+      <c r="O52" s="58">
+        <f>O16</f>
+      </c>
+      <c r="P52" s="25">
         <f>SUM(D52:O52)</f>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B53" s="55" t="s">
+      <c r="B53" s="56" t="s">
         <v>118</v>
       </c>
-      <c r="C53" s="56" t="s">
+      <c r="C53" s="57" t="s">
         <v>119</v>
       </c>
       <c r="D53" s="59">
@@ -3743,44 +3743,44 @@
       <c r="B54" s="60" t="s">
         <v>120</v>
       </c>
-      <c r="C54" s="56" t="s">
+      <c r="C54" s="57" t="s">
         <v>121</v>
       </c>
       <c r="D54" s="61">
-        <f>D53+D14+D15+D16</f>
+        <f>D53+D14*Configuración!$C$27+D15*Configuración!$C$28+D16*Configuración!$C$31</f>
       </c>
       <c r="E54" s="61">
-        <f>E53+E14+E15+E16</f>
+        <f>E53+E14*Configuración!$C$27+E15*Configuración!$C$28+E16*Configuración!$C$31</f>
       </c>
       <c r="F54" s="61">
-        <f>F53+F14+F15+F16</f>
+        <f>F53+F14*Configuración!$C$27+F15*Configuración!$C$28+F16*Configuración!$C$31</f>
       </c>
       <c r="G54" s="61">
-        <f>G53+G14+G15+G16</f>
+        <f>G53+G14*Configuración!$C$27+G15*Configuración!$C$28+G16*Configuración!$C$31</f>
       </c>
       <c r="H54" s="61">
-        <f>H53+H14+H15+H16</f>
+        <f>H53+H14*Configuración!$C$27+H15*Configuración!$C$28+H16*Configuración!$C$31</f>
       </c>
       <c r="I54" s="61">
-        <f>I53+I14+I15+I16</f>
+        <f>I53+I14*Configuración!$C$27+I15*Configuración!$C$28+I16*Configuración!$C$31</f>
       </c>
       <c r="J54" s="61">
-        <f>J53+J14+J15+J16</f>
+        <f>J53+J14*Configuración!$C$27+J15*Configuración!$C$28+J16*Configuración!$C$31</f>
       </c>
       <c r="K54" s="61">
-        <f>K53+K14+K15+K16</f>
+        <f>K53+K14*Configuración!$C$27+K15*Configuración!$C$28+K16*Configuración!$C$31</f>
       </c>
       <c r="L54" s="61">
-        <f>L53+L14+L15+L16</f>
+        <f>L53+L14*Configuración!$C$27+L15*Configuración!$C$28+L16*Configuración!$C$31</f>
       </c>
       <c r="M54" s="61">
-        <f>M53+M14+M15+M16</f>
+        <f>M53+M14*Configuración!$C$27+M15*Configuración!$C$28+M16*Configuración!$C$31</f>
       </c>
       <c r="N54" s="61">
-        <f>N53+N14+N15+N16</f>
+        <f>N53+N14*Configuración!$C$27+N15*Configuración!$C$28+N16*Configuración!$C$31</f>
       </c>
       <c r="O54" s="61">
-        <f>O53+O14+O15+O16</f>
+        <f>O53+O14*Configuración!$C$27+O15*Configuración!$C$28+O16*Configuración!$C$31</f>
       </c>
       <c r="P54" s="61">
         <f>SUM(D54:O54)</f>
@@ -3852,24 +3852,24 @@
       <c r="P56" s="2"/>
     </row>
     <row r="57" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A57" s="54" t="s">
+      <c r="A57" s="55" t="s">
         <v>124</v>
       </c>
-      <c r="B57" s="54"/>
-      <c r="C57" s="54"/>
-      <c r="D57" s="54"/>
-      <c r="E57" s="54"/>
-      <c r="F57" s="54"/>
-      <c r="G57" s="54"/>
-      <c r="H57" s="54"/>
-      <c r="I57" s="54"/>
-      <c r="J57" s="54"/>
-      <c r="K57" s="54"/>
-      <c r="L57" s="54"/>
-      <c r="M57" s="54"/>
-      <c r="N57" s="54"/>
-      <c r="O57" s="54"/>
-      <c r="P57" s="54"/>
+      <c r="B57" s="55"/>
+      <c r="C57" s="55"/>
+      <c r="D57" s="55"/>
+      <c r="E57" s="55"/>
+      <c r="F57" s="55"/>
+      <c r="G57" s="55"/>
+      <c r="H57" s="55"/>
+      <c r="I57" s="55"/>
+      <c r="J57" s="55"/>
+      <c r="K57" s="55"/>
+      <c r="L57" s="55"/>
+      <c r="M57" s="55"/>
+      <c r="N57" s="55"/>
+      <c r="O57" s="55"/>
+      <c r="P57" s="55"/>
     </row>
     <row r="58" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" s="65" t="s">

</xml_diff>

<commit_message>
Fix: quantity inputs for variable rows, update section header, fix undefined color
- Variable rows now show (horas)/(días) labels and accept quantities
- Section header updated to clarify quantity vs euro input
- Fix C.verdeSuave undefined reference → C.vs

https://claude.ai/code/session_01WLGGf5vt4LjNM5wLNiuW4q
</commit_message>
<xml_diff>
--- a/calculadora-nomina-v3.xlsx
+++ b/calculadora-nomina-v3.xlsx
@@ -215,7 +215,7 @@
     <t>↑ edita cada mes</t>
   </si>
   <si>
-    <t>📋  DEVENGOS — Las celdas amarillas son editables. Introduce el importe en €.</t>
+    <t>📋  DEVENGOS — Celdas amarillas editables. Variables (horas/días/km): introduce CANTIDADES. Salario, Actividad, Dieta y Paga Extra: introduce €.</t>
   </si>
   <si>
     <t>Salario Convenio</t>
@@ -680,13 +680,13 @@
     </font>
     <font>
       <b/>
-      <color rgb="0F172A"/>
+      <color rgb="065F46"/>
       <sz val="10"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="0F172A"/>
+      <color rgb="065F46"/>
       <sz val="14"/>
       <name val="Calibri"/>
     </font>

</xml_diff>

<commit_message>
Fix formula bugs: DIAF no suma a bruto, doble conteo en TOT7P, visibilidad paga extra
- Días fuera España (DIAF) es ahora puro contador para Art.7p: NO multiplica
  por precio y NO suma al Bruto Sujeto mensual ni a la Base CC.
  La compensación económica por días fuera va en Dieta (exento) y
  H.Desplazamiento, no en un concepto de días separado.
- TOT7P eliminaba doble conteo: PROP7P ya captura el salario proporcional
  a los días fuera; añadir DIAF×PDIAF encima era contar esos días dos veces.
- Etiqueta DIAF actualizada a 'contador 7p'; total columna muestra días (NUM)
- Sección TOTALES y nota al pie aclaradas: Bruto Sujeto es sin paga extra,
  la paga extra sí suma en el BRUTO ANUAL del resumen final.

https://claude.ai/code/session_01WLGGf5vt4LjNM5wLNiuW4q
</commit_message>
<xml_diff>
--- a/calculadora-nomina-v3.xlsx
+++ b/calculadora-nomina-v3.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="137">
   <si>
     <t>⚙️  CONFIGURACIÓN — Nómina 2026</t>
   </si>
@@ -143,10 +143,10 @@
     <t>HHEE</t>
   </si>
   <si>
-    <t>Días fuera (bruto/día)</t>
-  </si>
-  <si>
-    <t>Base CC + Art.7p  ← = C6</t>
+    <t>Días fuera (precio/día ref.)</t>
+  </si>
+  <si>
+    <t>Ref. informativa ← = C6 (no suma a devengos; solo para referencia del valor diario)</t>
   </si>
   <si>
     <t>KM</t>
@@ -251,7 +251,10 @@
     <t>H. Desp. Festivo (horas)</t>
   </si>
   <si>
-    <t>Días fuera (días)</t>
+    <t>Días fuera España (días)</t>
+  </si>
+  <si>
+    <t>contador 7p</t>
   </si>
   <si>
     <t>H. Extra Normal (horas)</t>
@@ -287,7 +290,7 @@
     <t>PAGA EXTRA</t>
   </si>
   <si>
-    <t>🔢  TOTALES CALCULADOS</t>
+    <t>🔢  TOTALES CALCULADOS  ·  Bruto Sujeto = devengos del mes sin paga extra  ·  Paga extra ⭐ aparece en su sección propia y se suma en el RESUMEN ANUAL al pie de la hoja</t>
   </si>
   <si>
     <t>Bruto Sujeto (base IRPF)</t>
@@ -377,7 +380,7 @@
     <t>7p</t>
   </si>
   <si>
-    <t>Renta 7p (prop.sal + desp + días fuera €)</t>
+    <t>Renta 7p (salario prop. días fuera + desplazamiento)</t>
   </si>
   <si>
     <t>7p TOTAL</t>
@@ -404,7 +407,7 @@
     <t>IRPF retenido total a recuperar en la Renta</t>
   </si>
   <si>
-    <t>⚠️  Celdas amarillas = editables  |  IRPF editable por mes (fila "IRPF %")  |  Art.7p requiere trabajo físico en el extranjero y país destino con IRPF equivalente; consulta con gestor  |  Paga extra ⭐ = normalmente junio y diciembre; ponla en la fila "Paga Extra €" del mes correspondiente</t>
+    <t>⚠️  Celdas amarillas = editables  |  IRPF editable por mes (fila "IRPF %")  |  Días fuera España = introduce NÚMERO DE DÍAS (solo cuenta para Art.7p; NO suma al bruto mensual, la paga por estar fuera va en Dieta/Desplazamiento)  |  Paga extra ⭐ = ponla en junio/diciembre; el "Bruto Sujeto" del mes NO la incluye pero el BRUTO ANUAL del resumen inferior SÍ la suma  |  Art.7p: requiere trabajo físico fuera de España; consulta con gestor</t>
   </si>
   <si>
     <t>📊  RESUMEN ANUAL — Bruto y Neto total (con variables) vs Solo salario fijo (sin variables)</t>
@@ -811,7 +814,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -885,6 +888,9 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="15" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2344,7 +2350,7 @@
         <v>78</v>
       </c>
       <c r="C16" s="27" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D16" s="26">
         <v>0</v>
@@ -2382,16 +2388,16 @@
       <c r="O16" s="26">
         <v>0</v>
       </c>
-      <c r="P16" s="25">
-        <f>SUM(D16:O16)*Configuración!$C$31</f>
+      <c r="P16" s="28">
+        <f>SUM(D16:O16)</f>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B17" s="22" t="s">
-        <v>79</v>
-      </c>
-      <c r="C17" s="28" t="s">
         <v>80</v>
+      </c>
+      <c r="C17" s="29" t="s">
+        <v>81</v>
       </c>
       <c r="D17" s="26">
         <v>0</v>
@@ -2435,9 +2441,9 @@
     </row>
     <row r="18" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B18" s="22" t="s">
-        <v>81</v>
-      </c>
-      <c r="C18" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="C18" s="29" t="s">
         <v>41</v>
       </c>
       <c r="D18" s="26">
@@ -2499,31 +2505,31 @@
       <c r="P19" s="20"/>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A20" s="29" t="s">
-        <v>82</v>
-      </c>
-      <c r="B20" s="29"/>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="29"/>
-      <c r="G20" s="29"/>
-      <c r="H20" s="29"/>
-      <c r="I20" s="29"/>
-      <c r="J20" s="29"/>
-      <c r="K20" s="29"/>
-      <c r="L20" s="29"/>
-      <c r="M20" s="29"/>
-      <c r="N20" s="29"/>
-      <c r="O20" s="29"/>
-      <c r="P20" s="29"/>
+      <c r="A20" s="30" t="s">
+        <v>83</v>
+      </c>
+      <c r="B20" s="30"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="30"/>
+      <c r="H20" s="30"/>
+      <c r="I20" s="30"/>
+      <c r="J20" s="30"/>
+      <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
+      <c r="M20" s="30"/>
+      <c r="N20" s="30"/>
+      <c r="O20" s="30"/>
+      <c r="P20" s="30"/>
     </row>
     <row r="21" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B21" s="30" t="s">
-        <v>83</v>
-      </c>
-      <c r="C21" s="31" t="s">
+      <c r="B21" s="31" t="s">
         <v>84</v>
+      </c>
+      <c r="C21" s="32" t="s">
+        <v>85</v>
       </c>
       <c r="D21" s="6">
         <v>0</v>
@@ -2566,11 +2572,11 @@
       </c>
     </row>
     <row r="22" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B22" s="30" t="s">
+      <c r="B22" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="C22" s="32" t="s">
         <v>85</v>
-      </c>
-      <c r="C22" s="31" t="s">
-        <v>84</v>
       </c>
       <c r="D22" s="6">
         <v>0</v>
@@ -2613,11 +2619,11 @@
       </c>
     </row>
     <row r="23" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B23" s="30" t="s">
-        <v>86</v>
-      </c>
-      <c r="C23" s="31" t="s">
-        <v>84</v>
+      <c r="B23" s="31" t="s">
+        <v>87</v>
+      </c>
+      <c r="C23" s="32" t="s">
+        <v>85</v>
       </c>
       <c r="D23" s="26">
         <v>0</v>
@@ -2678,31 +2684,31 @@
       <c r="P24" s="20"/>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A25" s="32" t="s">
-        <v>87</v>
-      </c>
-      <c r="B25" s="32"/>
-      <c r="C25" s="32"/>
-      <c r="D25" s="32"/>
-      <c r="E25" s="32"/>
-      <c r="F25" s="32"/>
-      <c r="G25" s="32"/>
-      <c r="H25" s="32"/>
-      <c r="I25" s="32"/>
-      <c r="J25" s="32"/>
-      <c r="K25" s="32"/>
-      <c r="L25" s="32"/>
-      <c r="M25" s="32"/>
-      <c r="N25" s="32"/>
-      <c r="O25" s="32"/>
-      <c r="P25" s="32"/>
+      <c r="A25" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="B25" s="33"/>
+      <c r="C25" s="33"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="33"/>
+      <c r="G25" s="33"/>
+      <c r="H25" s="33"/>
+      <c r="I25" s="33"/>
+      <c r="J25" s="33"/>
+      <c r="K25" s="33"/>
+      <c r="L25" s="33"/>
+      <c r="M25" s="33"/>
+      <c r="N25" s="33"/>
+      <c r="O25" s="33"/>
+      <c r="P25" s="33"/>
     </row>
     <row r="26" ht="20" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B26" s="33" t="s">
-        <v>88</v>
-      </c>
-      <c r="C26" s="34" t="s">
+      <c r="B26" s="34" t="s">
         <v>89</v>
+      </c>
+      <c r="C26" s="35" t="s">
+        <v>90</v>
       </c>
       <c r="D26" s="6">
         <v>0</v>
@@ -2764,7 +2770,7 @@
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -2783,93 +2789,93 @@
       <c r="P28" s="3"/>
     </row>
     <row r="29" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B29" s="35" t="s">
-        <v>91</v>
-      </c>
-      <c r="C29" s="36" t="s">
+      <c r="B29" s="36" t="s">
         <v>92</v>
       </c>
-      <c r="D29" s="37">
-        <f>D7+D8+D9*Configuración!$C$22+D10*Configuración!$C$23+D11*Configuración!$C$24+D12*Configuración!$C$25+D13*Configuración!$C$26+D14*Configuración!$C$27+D15*Configuración!$C$28+D16*Configuración!$C$31+D17*Configuración!$C$29+D18*Configuración!$C$30</f>
-      </c>
-      <c r="E29" s="37">
-        <f>E7+E8+E9*Configuración!$C$22+E10*Configuración!$C$23+E11*Configuración!$C$24+E12*Configuración!$C$25+E13*Configuración!$C$26+E14*Configuración!$C$27+E15*Configuración!$C$28+E16*Configuración!$C$31+E17*Configuración!$C$29+E18*Configuración!$C$30</f>
-      </c>
-      <c r="F29" s="37">
-        <f>F7+F8+F9*Configuración!$C$22+F10*Configuración!$C$23+F11*Configuración!$C$24+F12*Configuración!$C$25+F13*Configuración!$C$26+F14*Configuración!$C$27+F15*Configuración!$C$28+F16*Configuración!$C$31+F17*Configuración!$C$29+F18*Configuración!$C$30</f>
-      </c>
-      <c r="G29" s="37">
-        <f>G7+G8+G9*Configuración!$C$22+G10*Configuración!$C$23+G11*Configuración!$C$24+G12*Configuración!$C$25+G13*Configuración!$C$26+G14*Configuración!$C$27+G15*Configuración!$C$28+G16*Configuración!$C$31+G17*Configuración!$C$29+G18*Configuración!$C$30</f>
-      </c>
-      <c r="H29" s="37">
-        <f>H7+H8+H9*Configuración!$C$22+H10*Configuración!$C$23+H11*Configuración!$C$24+H12*Configuración!$C$25+H13*Configuración!$C$26+H14*Configuración!$C$27+H15*Configuración!$C$28+H16*Configuración!$C$31+H17*Configuración!$C$29+H18*Configuración!$C$30</f>
-      </c>
-      <c r="I29" s="37">
-        <f>I7+I8+I9*Configuración!$C$22+I10*Configuración!$C$23+I11*Configuración!$C$24+I12*Configuración!$C$25+I13*Configuración!$C$26+I14*Configuración!$C$27+I15*Configuración!$C$28+I16*Configuración!$C$31+I17*Configuración!$C$29+I18*Configuración!$C$30</f>
-      </c>
-      <c r="J29" s="37">
-        <f>J7+J8+J9*Configuración!$C$22+J10*Configuración!$C$23+J11*Configuración!$C$24+J12*Configuración!$C$25+J13*Configuración!$C$26+J14*Configuración!$C$27+J15*Configuración!$C$28+J16*Configuración!$C$31+J17*Configuración!$C$29+J18*Configuración!$C$30</f>
-      </c>
-      <c r="K29" s="37">
-        <f>K7+K8+K9*Configuración!$C$22+K10*Configuración!$C$23+K11*Configuración!$C$24+K12*Configuración!$C$25+K13*Configuración!$C$26+K14*Configuración!$C$27+K15*Configuración!$C$28+K16*Configuración!$C$31+K17*Configuración!$C$29+K18*Configuración!$C$30</f>
-      </c>
-      <c r="L29" s="37">
-        <f>L7+L8+L9*Configuración!$C$22+L10*Configuración!$C$23+L11*Configuración!$C$24+L12*Configuración!$C$25+L13*Configuración!$C$26+L14*Configuración!$C$27+L15*Configuración!$C$28+L16*Configuración!$C$31+L17*Configuración!$C$29+L18*Configuración!$C$30</f>
-      </c>
-      <c r="M29" s="37">
-        <f>M7+M8+M9*Configuración!$C$22+M10*Configuración!$C$23+M11*Configuración!$C$24+M12*Configuración!$C$25+M13*Configuración!$C$26+M14*Configuración!$C$27+M15*Configuración!$C$28+M16*Configuración!$C$31+M17*Configuración!$C$29+M18*Configuración!$C$30</f>
-      </c>
-      <c r="N29" s="37">
-        <f>N7+N8+N9*Configuración!$C$22+N10*Configuración!$C$23+N11*Configuración!$C$24+N12*Configuración!$C$25+N13*Configuración!$C$26+N14*Configuración!$C$27+N15*Configuración!$C$28+N16*Configuración!$C$31+N17*Configuración!$C$29+N18*Configuración!$C$30</f>
-      </c>
-      <c r="O29" s="37">
-        <f>O7+O8+O9*Configuración!$C$22+O10*Configuración!$C$23+O11*Configuración!$C$24+O12*Configuración!$C$25+O13*Configuración!$C$26+O14*Configuración!$C$27+O15*Configuración!$C$28+O16*Configuración!$C$31+O17*Configuración!$C$29+O18*Configuración!$C$30</f>
-      </c>
-      <c r="P29" s="37">
+      <c r="C29" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="D29" s="38">
+        <f>D7+D8+D9*Configuración!$C$22+D10*Configuración!$C$23+D11*Configuración!$C$24+D12*Configuración!$C$25+D13*Configuración!$C$26+D14*Configuración!$C$27+D15*Configuración!$C$28+D17*Configuración!$C$29+D18*Configuración!$C$30</f>
+      </c>
+      <c r="E29" s="38">
+        <f>E7+E8+E9*Configuración!$C$22+E10*Configuración!$C$23+E11*Configuración!$C$24+E12*Configuración!$C$25+E13*Configuración!$C$26+E14*Configuración!$C$27+E15*Configuración!$C$28+E17*Configuración!$C$29+E18*Configuración!$C$30</f>
+      </c>
+      <c r="F29" s="38">
+        <f>F7+F8+F9*Configuración!$C$22+F10*Configuración!$C$23+F11*Configuración!$C$24+F12*Configuración!$C$25+F13*Configuración!$C$26+F14*Configuración!$C$27+F15*Configuración!$C$28+F17*Configuración!$C$29+F18*Configuración!$C$30</f>
+      </c>
+      <c r="G29" s="38">
+        <f>G7+G8+G9*Configuración!$C$22+G10*Configuración!$C$23+G11*Configuración!$C$24+G12*Configuración!$C$25+G13*Configuración!$C$26+G14*Configuración!$C$27+G15*Configuración!$C$28+G17*Configuración!$C$29+G18*Configuración!$C$30</f>
+      </c>
+      <c r="H29" s="38">
+        <f>H7+H8+H9*Configuración!$C$22+H10*Configuración!$C$23+H11*Configuración!$C$24+H12*Configuración!$C$25+H13*Configuración!$C$26+H14*Configuración!$C$27+H15*Configuración!$C$28+H17*Configuración!$C$29+H18*Configuración!$C$30</f>
+      </c>
+      <c r="I29" s="38">
+        <f>I7+I8+I9*Configuración!$C$22+I10*Configuración!$C$23+I11*Configuración!$C$24+I12*Configuración!$C$25+I13*Configuración!$C$26+I14*Configuración!$C$27+I15*Configuración!$C$28+I17*Configuración!$C$29+I18*Configuración!$C$30</f>
+      </c>
+      <c r="J29" s="38">
+        <f>J7+J8+J9*Configuración!$C$22+J10*Configuración!$C$23+J11*Configuración!$C$24+J12*Configuración!$C$25+J13*Configuración!$C$26+J14*Configuración!$C$27+J15*Configuración!$C$28+J17*Configuración!$C$29+J18*Configuración!$C$30</f>
+      </c>
+      <c r="K29" s="38">
+        <f>K7+K8+K9*Configuración!$C$22+K10*Configuración!$C$23+K11*Configuración!$C$24+K12*Configuración!$C$25+K13*Configuración!$C$26+K14*Configuración!$C$27+K15*Configuración!$C$28+K17*Configuración!$C$29+K18*Configuración!$C$30</f>
+      </c>
+      <c r="L29" s="38">
+        <f>L7+L8+L9*Configuración!$C$22+L10*Configuración!$C$23+L11*Configuración!$C$24+L12*Configuración!$C$25+L13*Configuración!$C$26+L14*Configuración!$C$27+L15*Configuración!$C$28+L17*Configuración!$C$29+L18*Configuración!$C$30</f>
+      </c>
+      <c r="M29" s="38">
+        <f>M7+M8+M9*Configuración!$C$22+M10*Configuración!$C$23+M11*Configuración!$C$24+M12*Configuración!$C$25+M13*Configuración!$C$26+M14*Configuración!$C$27+M15*Configuración!$C$28+M17*Configuración!$C$29+M18*Configuración!$C$30</f>
+      </c>
+      <c r="N29" s="38">
+        <f>N7+N8+N9*Configuración!$C$22+N10*Configuración!$C$23+N11*Configuración!$C$24+N12*Configuración!$C$25+N13*Configuración!$C$26+N14*Configuración!$C$27+N15*Configuración!$C$28+N17*Configuración!$C$29+N18*Configuración!$C$30</f>
+      </c>
+      <c r="O29" s="38">
+        <f>O7+O8+O9*Configuración!$C$22+O10*Configuración!$C$23+O11*Configuración!$C$24+O12*Configuración!$C$25+O13*Configuración!$C$26+O14*Configuración!$C$27+O15*Configuración!$C$28+O17*Configuración!$C$29+O18*Configuración!$C$30</f>
+      </c>
+      <c r="P29" s="38">
         <f>SUM(D29:O29)</f>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B30" s="38" t="s">
-        <v>93</v>
+      <c r="B30" s="39" t="s">
+        <v>94</v>
       </c>
       <c r="C30" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="D30" s="39">
+        <v>95</v>
+      </c>
+      <c r="D30" s="40">
         <f>D17*Configuración!$C$29+D18*Configuración!$C$30</f>
       </c>
-      <c r="E30" s="39">
+      <c r="E30" s="40">
         <f>E17*Configuración!$C$29+E18*Configuración!$C$30</f>
       </c>
-      <c r="F30" s="39">
+      <c r="F30" s="40">
         <f>F17*Configuración!$C$29+F18*Configuración!$C$30</f>
       </c>
-      <c r="G30" s="39">
+      <c r="G30" s="40">
         <f>G17*Configuración!$C$29+G18*Configuración!$C$30</f>
       </c>
-      <c r="H30" s="39">
+      <c r="H30" s="40">
         <f>H17*Configuración!$C$29+H18*Configuración!$C$30</f>
       </c>
-      <c r="I30" s="39">
+      <c r="I30" s="40">
         <f>I17*Configuración!$C$29+I18*Configuración!$C$30</f>
       </c>
-      <c r="J30" s="39">
+      <c r="J30" s="40">
         <f>J17*Configuración!$C$29+J18*Configuración!$C$30</f>
       </c>
-      <c r="K30" s="39">
+      <c r="K30" s="40">
         <f>K17*Configuración!$C$29+K18*Configuración!$C$30</f>
       </c>
-      <c r="L30" s="39">
+      <c r="L30" s="40">
         <f>L17*Configuración!$C$29+L18*Configuración!$C$30</f>
       </c>
-      <c r="M30" s="39">
+      <c r="M30" s="40">
         <f>M17*Configuración!$C$29+M18*Configuración!$C$30</f>
       </c>
-      <c r="N30" s="39">
+      <c r="N30" s="40">
         <f>N17*Configuración!$C$29+N18*Configuración!$C$30</f>
       </c>
-      <c r="O30" s="39">
+      <c r="O30" s="40">
         <f>O17*Configuración!$C$29+O18*Configuración!$C$30</f>
       </c>
       <c r="P30" s="25">
@@ -2877,46 +2883,46 @@
       </c>
     </row>
     <row r="31" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B31" s="30" t="s">
-        <v>95</v>
-      </c>
-      <c r="C31" s="31" t="s">
-        <v>84</v>
-      </c>
-      <c r="D31" s="40">
+      <c r="B31" s="31" t="s">
+        <v>96</v>
+      </c>
+      <c r="C31" s="32" t="s">
+        <v>85</v>
+      </c>
+      <c r="D31" s="41">
         <f>D21+D22+D23*Configuración!$C$32</f>
       </c>
-      <c r="E31" s="40">
+      <c r="E31" s="41">
         <f>E21+E22+E23*Configuración!$C$32</f>
       </c>
-      <c r="F31" s="40">
+      <c r="F31" s="41">
         <f>F21+F22+F23*Configuración!$C$32</f>
       </c>
-      <c r="G31" s="40">
+      <c r="G31" s="41">
         <f>G21+G22+G23*Configuración!$C$32</f>
       </c>
-      <c r="H31" s="40">
+      <c r="H31" s="41">
         <f>H21+H22+H23*Configuración!$C$32</f>
       </c>
-      <c r="I31" s="40">
+      <c r="I31" s="41">
         <f>I21+I22+I23*Configuración!$C$32</f>
       </c>
-      <c r="J31" s="40">
+      <c r="J31" s="41">
         <f>J21+J22+J23*Configuración!$C$32</f>
       </c>
-      <c r="K31" s="40">
+      <c r="K31" s="41">
         <f>K21+K22+K23*Configuración!$C$32</f>
       </c>
-      <c r="L31" s="40">
+      <c r="L31" s="41">
         <f>L21+L22+L23*Configuración!$C$32</f>
       </c>
-      <c r="M31" s="40">
+      <c r="M31" s="41">
         <f>M21+M22+M23*Configuración!$C$32</f>
       </c>
-      <c r="N31" s="40">
+      <c r="N31" s="41">
         <f>N21+N22+N23*Configuración!$C$32</f>
       </c>
-      <c r="O31" s="40">
+      <c r="O31" s="41">
         <f>O21+O22+O23*Configuración!$C$32</f>
       </c>
       <c r="P31" s="25">
@@ -2942,63 +2948,63 @@
       <c r="P32" s="20"/>
     </row>
     <row r="33" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A33" s="41" t="s">
-        <v>96</v>
-      </c>
-      <c r="B33" s="41"/>
-      <c r="C33" s="41"/>
-      <c r="D33" s="41"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="41"/>
-      <c r="G33" s="41"/>
-      <c r="H33" s="41"/>
-      <c r="I33" s="41"/>
-      <c r="J33" s="41"/>
-      <c r="K33" s="41"/>
-      <c r="L33" s="41"/>
-      <c r="M33" s="41"/>
-      <c r="N33" s="41"/>
-      <c r="O33" s="41"/>
-      <c r="P33" s="41"/>
+      <c r="A33" s="42" t="s">
+        <v>97</v>
+      </c>
+      <c r="B33" s="42"/>
+      <c r="C33" s="42"/>
+      <c r="D33" s="42"/>
+      <c r="E33" s="42"/>
+      <c r="F33" s="42"/>
+      <c r="G33" s="42"/>
+      <c r="H33" s="42"/>
+      <c r="I33" s="42"/>
+      <c r="J33" s="42"/>
+      <c r="K33" s="42"/>
+      <c r="L33" s="42"/>
+      <c r="M33" s="42"/>
+      <c r="N33" s="42"/>
+      <c r="O33" s="42"/>
+      <c r="P33" s="42"/>
     </row>
     <row r="34" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B34" s="42" t="s">
-        <v>97</v>
-      </c>
-      <c r="D34" s="43">
+      <c r="B34" s="43" t="s">
+        <v>98</v>
+      </c>
+      <c r="D34" s="44">
         <f>D29-D30+Configuración!$C$7</f>
       </c>
-      <c r="E34" s="43">
+      <c r="E34" s="44">
         <f>E29-E30+Configuración!$C$7</f>
       </c>
-      <c r="F34" s="43">
+      <c r="F34" s="44">
         <f>F29-F30+Configuración!$C$7</f>
       </c>
-      <c r="G34" s="43">
+      <c r="G34" s="44">
         <f>G29-G30+Configuración!$C$7</f>
       </c>
-      <c r="H34" s="43">
+      <c r="H34" s="44">
         <f>H29-H30+Configuración!$C$7</f>
       </c>
-      <c r="I34" s="43">
+      <c r="I34" s="44">
         <f>I29-I30+Configuración!$C$7</f>
       </c>
-      <c r="J34" s="43">
+      <c r="J34" s="44">
         <f>J29-J30+Configuración!$C$7</f>
       </c>
-      <c r="K34" s="43">
+      <c r="K34" s="44">
         <f>K29-K30+Configuración!$C$7</f>
       </c>
-      <c r="L34" s="43">
+      <c r="L34" s="44">
         <f>L29-L30+Configuración!$C$7</f>
       </c>
-      <c r="M34" s="43">
+      <c r="M34" s="44">
         <f>M29-M30+Configuración!$C$7</f>
       </c>
-      <c r="N34" s="43">
+      <c r="N34" s="44">
         <f>N29-N30+Configuración!$C$7</f>
       </c>
-      <c r="O34" s="43">
+      <c r="O34" s="44">
         <f>O29-O30+Configuración!$C$7</f>
       </c>
       <c r="P34" s="25">
@@ -3006,43 +3012,43 @@
       </c>
     </row>
     <row r="35" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B35" s="42" t="s">
+      <c r="B35" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="D35" s="43">
+      <c r="D35" s="44">
         <f>D34+D30</f>
       </c>
-      <c r="E35" s="43">
+      <c r="E35" s="44">
         <f>E34+E30</f>
       </c>
-      <c r="F35" s="43">
+      <c r="F35" s="44">
         <f>F34+F30</f>
       </c>
-      <c r="G35" s="43">
+      <c r="G35" s="44">
         <f>G34+G30</f>
       </c>
-      <c r="H35" s="43">
+      <c r="H35" s="44">
         <f>H34+H30</f>
       </c>
-      <c r="I35" s="43">
+      <c r="I35" s="44">
         <f>I34+I30</f>
       </c>
-      <c r="J35" s="43">
+      <c r="J35" s="44">
         <f>J34+J30</f>
       </c>
-      <c r="K35" s="43">
+      <c r="K35" s="44">
         <f>K34+K30</f>
       </c>
-      <c r="L35" s="43">
+      <c r="L35" s="44">
         <f>L34+L30</f>
       </c>
-      <c r="M35" s="43">
+      <c r="M35" s="44">
         <f>M34+M30</f>
       </c>
-      <c r="N35" s="43">
+      <c r="N35" s="44">
         <f>N34+N30</f>
       </c>
-      <c r="O35" s="43">
+      <c r="O35" s="44">
         <f>O34+O30</f>
       </c>
       <c r="P35" s="25">
@@ -3050,46 +3056,46 @@
       </c>
     </row>
     <row r="36" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B36" s="44" t="s">
-        <v>98</v>
-      </c>
-      <c r="C36" s="45" t="s">
+      <c r="B36" s="45" t="s">
         <v>99</v>
       </c>
-      <c r="D36" s="46">
+      <c r="C36" s="46" t="s">
+        <v>100</v>
+      </c>
+      <c r="D36" s="47">
         <f>D34*Configuración!$C$12</f>
       </c>
-      <c r="E36" s="46">
+      <c r="E36" s="47">
         <f>E34*Configuración!$C$12</f>
       </c>
-      <c r="F36" s="46">
+      <c r="F36" s="47">
         <f>F34*Configuración!$C$12</f>
       </c>
-      <c r="G36" s="46">
+      <c r="G36" s="47">
         <f>G34*Configuración!$C$12</f>
       </c>
-      <c r="H36" s="46">
+      <c r="H36" s="47">
         <f>H34*Configuración!$C$12</f>
       </c>
-      <c r="I36" s="46">
+      <c r="I36" s="47">
         <f>I34*Configuración!$C$12</f>
       </c>
-      <c r="J36" s="46">
+      <c r="J36" s="47">
         <f>J34*Configuración!$C$12</f>
       </c>
-      <c r="K36" s="46">
+      <c r="K36" s="47">
         <f>K34*Configuración!$C$12</f>
       </c>
-      <c r="L36" s="46">
+      <c r="L36" s="47">
         <f>L34*Configuración!$C$12</f>
       </c>
-      <c r="M36" s="46">
+      <c r="M36" s="47">
         <f>M34*Configuración!$C$12</f>
       </c>
-      <c r="N36" s="46">
+      <c r="N36" s="47">
         <f>N34*Configuración!$C$12</f>
       </c>
-      <c r="O36" s="46">
+      <c r="O36" s="47">
         <f>O34*Configuración!$C$12</f>
       </c>
       <c r="P36" s="25">
@@ -3097,46 +3103,46 @@
       </c>
     </row>
     <row r="37" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B37" s="44" t="s">
-        <v>100</v>
-      </c>
-      <c r="C37" s="45" t="s">
+      <c r="B37" s="45" t="s">
         <v>101</v>
       </c>
-      <c r="D37" s="46">
+      <c r="C37" s="46" t="s">
+        <v>102</v>
+      </c>
+      <c r="D37" s="47">
         <f>D35*Configuración!$C$13</f>
       </c>
-      <c r="E37" s="46">
+      <c r="E37" s="47">
         <f>E35*Configuración!$C$13</f>
       </c>
-      <c r="F37" s="46">
+      <c r="F37" s="47">
         <f>F35*Configuración!$C$13</f>
       </c>
-      <c r="G37" s="46">
+      <c r="G37" s="47">
         <f>G35*Configuración!$C$13</f>
       </c>
-      <c r="H37" s="46">
+      <c r="H37" s="47">
         <f>H35*Configuración!$C$13</f>
       </c>
-      <c r="I37" s="46">
+      <c r="I37" s="47">
         <f>I35*Configuración!$C$13</f>
       </c>
-      <c r="J37" s="46">
+      <c r="J37" s="47">
         <f>J35*Configuración!$C$13</f>
       </c>
-      <c r="K37" s="46">
+      <c r="K37" s="47">
         <f>K35*Configuración!$C$13</f>
       </c>
-      <c r="L37" s="46">
+      <c r="L37" s="47">
         <f>L35*Configuración!$C$13</f>
       </c>
-      <c r="M37" s="46">
+      <c r="M37" s="47">
         <f>M35*Configuración!$C$13</f>
       </c>
-      <c r="N37" s="46">
+      <c r="N37" s="47">
         <f>N35*Configuración!$C$13</f>
       </c>
-      <c r="O37" s="46">
+      <c r="O37" s="47">
         <f>O35*Configuración!$C$13</f>
       </c>
       <c r="P37" s="25">
@@ -3144,46 +3150,46 @@
       </c>
     </row>
     <row r="38" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B38" s="44" t="s">
-        <v>102</v>
-      </c>
-      <c r="C38" s="45" t="s">
-        <v>99</v>
-      </c>
-      <c r="D38" s="46">
+      <c r="B38" s="45" t="s">
+        <v>103</v>
+      </c>
+      <c r="C38" s="46" t="s">
+        <v>100</v>
+      </c>
+      <c r="D38" s="47">
         <f>D30*Configuración!$C$14</f>
       </c>
-      <c r="E38" s="46">
+      <c r="E38" s="47">
         <f>E30*Configuración!$C$14</f>
       </c>
-      <c r="F38" s="46">
+      <c r="F38" s="47">
         <f>F30*Configuración!$C$14</f>
       </c>
-      <c r="G38" s="46">
+      <c r="G38" s="47">
         <f>G30*Configuración!$C$14</f>
       </c>
-      <c r="H38" s="46">
+      <c r="H38" s="47">
         <f>H30*Configuración!$C$14</f>
       </c>
-      <c r="I38" s="46">
+      <c r="I38" s="47">
         <f>I30*Configuración!$C$14</f>
       </c>
-      <c r="J38" s="46">
+      <c r="J38" s="47">
         <f>J30*Configuración!$C$14</f>
       </c>
-      <c r="K38" s="46">
+      <c r="K38" s="47">
         <f>K30*Configuración!$C$14</f>
       </c>
-      <c r="L38" s="46">
+      <c r="L38" s="47">
         <f>L30*Configuración!$C$14</f>
       </c>
-      <c r="M38" s="46">
+      <c r="M38" s="47">
         <f>M30*Configuración!$C$14</f>
       </c>
-      <c r="N38" s="46">
+      <c r="N38" s="47">
         <f>N30*Configuración!$C$14</f>
       </c>
-      <c r="O38" s="46">
+      <c r="O38" s="47">
         <f>O30*Configuración!$C$14</f>
       </c>
       <c r="P38" s="25">
@@ -3191,46 +3197,46 @@
       </c>
     </row>
     <row r="39" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B39" s="44" t="s">
-        <v>103</v>
-      </c>
-      <c r="C39" s="45" t="s">
+      <c r="B39" s="45" t="s">
         <v>104</v>
       </c>
-      <c r="D39" s="46">
+      <c r="C39" s="46" t="s">
+        <v>105</v>
+      </c>
+      <c r="D39" s="47">
         <f>D35*Configuración!$C$15</f>
       </c>
-      <c r="E39" s="46">
+      <c r="E39" s="47">
         <f>E35*Configuración!$C$15</f>
       </c>
-      <c r="F39" s="46">
+      <c r="F39" s="47">
         <f>F35*Configuración!$C$15</f>
       </c>
-      <c r="G39" s="46">
+      <c r="G39" s="47">
         <f>G35*Configuración!$C$15</f>
       </c>
-      <c r="H39" s="46">
+      <c r="H39" s="47">
         <f>H35*Configuración!$C$15</f>
       </c>
-      <c r="I39" s="46">
+      <c r="I39" s="47">
         <f>I35*Configuración!$C$15</f>
       </c>
-      <c r="J39" s="46">
+      <c r="J39" s="47">
         <f>J35*Configuración!$C$15</f>
       </c>
-      <c r="K39" s="46">
+      <c r="K39" s="47">
         <f>K35*Configuración!$C$15</f>
       </c>
-      <c r="L39" s="46">
+      <c r="L39" s="47">
         <f>L35*Configuración!$C$15</f>
       </c>
-      <c r="M39" s="46">
+      <c r="M39" s="47">
         <f>M35*Configuración!$C$15</f>
       </c>
-      <c r="N39" s="46">
+      <c r="N39" s="47">
         <f>N35*Configuración!$C$15</f>
       </c>
-      <c r="O39" s="46">
+      <c r="O39" s="47">
         <f>O35*Configuración!$C$15</f>
       </c>
       <c r="P39" s="25">
@@ -3238,46 +3244,46 @@
       </c>
     </row>
     <row r="40" ht="22" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B40" s="47" t="s">
-        <v>105</v>
-      </c>
-      <c r="D40" s="48">
+      <c r="B40" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="D40" s="49">
         <f>D36+D37+D38+D39</f>
       </c>
-      <c r="E40" s="48">
+      <c r="E40" s="49">
         <f>E36+E37+E38+E39</f>
       </c>
-      <c r="F40" s="48">
+      <c r="F40" s="49">
         <f>F36+F37+F38+F39</f>
       </c>
-      <c r="G40" s="48">
+      <c r="G40" s="49">
         <f>G36+G37+G38+G39</f>
       </c>
-      <c r="H40" s="48">
+      <c r="H40" s="49">
         <f>H36+H37+H38+H39</f>
       </c>
-      <c r="I40" s="48">
+      <c r="I40" s="49">
         <f>I36+I37+I38+I39</f>
       </c>
-      <c r="J40" s="48">
+      <c r="J40" s="49">
         <f>J36+J37+J38+J39</f>
       </c>
-      <c r="K40" s="48">
+      <c r="K40" s="49">
         <f>K36+K37+K38+K39</f>
       </c>
-      <c r="L40" s="48">
+      <c r="L40" s="49">
         <f>L36+L37+L38+L39</f>
       </c>
-      <c r="M40" s="48">
+      <c r="M40" s="49">
         <f>M36+M37+M38+M39</f>
       </c>
-      <c r="N40" s="48">
+      <c r="N40" s="49">
         <f>N36+N37+N38+N39</f>
       </c>
-      <c r="O40" s="48">
+      <c r="O40" s="49">
         <f>O36+O37+O38+O39</f>
       </c>
-      <c r="P40" s="48">
+      <c r="P40" s="49">
         <f>SUM(D40:O40)</f>
       </c>
     </row>
@@ -3300,63 +3306,63 @@
       <c r="P41" s="20"/>
     </row>
     <row r="42" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A42" s="32" t="s">
-        <v>106</v>
-      </c>
-      <c r="B42" s="32"/>
-      <c r="C42" s="32"/>
-      <c r="D42" s="32"/>
-      <c r="E42" s="32"/>
-      <c r="F42" s="32"/>
-      <c r="G42" s="32"/>
-      <c r="H42" s="32"/>
-      <c r="I42" s="32"/>
-      <c r="J42" s="32"/>
-      <c r="K42" s="32"/>
-      <c r="L42" s="32"/>
-      <c r="M42" s="32"/>
-      <c r="N42" s="32"/>
-      <c r="O42" s="32"/>
-      <c r="P42" s="32"/>
+      <c r="A42" s="33" t="s">
+        <v>107</v>
+      </c>
+      <c r="B42" s="33"/>
+      <c r="C42" s="33"/>
+      <c r="D42" s="33"/>
+      <c r="E42" s="33"/>
+      <c r="F42" s="33"/>
+      <c r="G42" s="33"/>
+      <c r="H42" s="33"/>
+      <c r="I42" s="33"/>
+      <c r="J42" s="33"/>
+      <c r="K42" s="33"/>
+      <c r="L42" s="33"/>
+      <c r="M42" s="33"/>
+      <c r="N42" s="33"/>
+      <c r="O42" s="33"/>
+      <c r="P42" s="33"/>
     </row>
     <row r="43" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B43" s="33" t="s">
-        <v>107</v>
-      </c>
-      <c r="D43" s="49">
+      <c r="B43" s="34" t="s">
+        <v>108</v>
+      </c>
+      <c r="D43" s="50">
         <f>D26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="E43" s="49">
+      <c r="E43" s="50">
         <f>E26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="F43" s="49">
+      <c r="F43" s="50">
         <f>F26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="G43" s="49">
+      <c r="G43" s="50">
         <f>G26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="H43" s="49">
+      <c r="H43" s="50">
         <f>H26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="I43" s="49">
+      <c r="I43" s="50">
         <f>I26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="J43" s="49">
+      <c r="J43" s="50">
         <f>J26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="K43" s="49">
+      <c r="K43" s="50">
         <f>K26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="L43" s="49">
+      <c r="L43" s="50">
         <f>L26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="M43" s="49">
+      <c r="M43" s="50">
         <f>M26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="N43" s="49">
+      <c r="N43" s="50">
         <f>N26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
-      <c r="O43" s="49">
+      <c r="O43" s="50">
         <f>O26*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)</f>
       </c>
       <c r="P43" s="25">
@@ -3364,43 +3370,43 @@
       </c>
     </row>
     <row r="44" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B44" s="33" t="s">
-        <v>108</v>
-      </c>
-      <c r="D44" s="49">
+      <c r="B44" s="34" t="s">
+        <v>109</v>
+      </c>
+      <c r="D44" s="50">
         <f>D26*D4</f>
       </c>
-      <c r="E44" s="49">
+      <c r="E44" s="50">
         <f>E26*E4</f>
       </c>
-      <c r="F44" s="49">
+      <c r="F44" s="50">
         <f>F26*F4</f>
       </c>
-      <c r="G44" s="49">
+      <c r="G44" s="50">
         <f>G26*G4</f>
       </c>
-      <c r="H44" s="49">
+      <c r="H44" s="50">
         <f>H26*H4</f>
       </c>
-      <c r="I44" s="49">
+      <c r="I44" s="50">
         <f>I26*I4</f>
       </c>
-      <c r="J44" s="49">
+      <c r="J44" s="50">
         <f>J26*J4</f>
       </c>
-      <c r="K44" s="49">
+      <c r="K44" s="50">
         <f>K26*K4</f>
       </c>
-      <c r="L44" s="49">
+      <c r="L44" s="50">
         <f>L26*L4</f>
       </c>
-      <c r="M44" s="49">
+      <c r="M44" s="50">
         <f>M26*M4</f>
       </c>
-      <c r="N44" s="49">
+      <c r="N44" s="50">
         <f>N26*N4</f>
       </c>
-      <c r="O44" s="49">
+      <c r="O44" s="50">
         <f>O26*O4</f>
       </c>
       <c r="P44" s="25">
@@ -3408,46 +3414,46 @@
       </c>
     </row>
     <row r="45" ht="20" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B45" s="50" t="s">
-        <v>109</v>
-      </c>
-      <c r="D45" s="51">
+      <c r="B45" s="51" t="s">
+        <v>110</v>
+      </c>
+      <c r="D45" s="52">
         <f>D26-D43-D44</f>
       </c>
-      <c r="E45" s="51">
+      <c r="E45" s="52">
         <f>E26-E43-E44</f>
       </c>
-      <c r="F45" s="51">
+      <c r="F45" s="52">
         <f>F26-F43-F44</f>
       </c>
-      <c r="G45" s="51">
+      <c r="G45" s="52">
         <f>G26-G43-G44</f>
       </c>
-      <c r="H45" s="51">
+      <c r="H45" s="52">
         <f>H26-H43-H44</f>
       </c>
-      <c r="I45" s="51">
+      <c r="I45" s="52">
         <f>I26-I43-I44</f>
       </c>
-      <c r="J45" s="51">
+      <c r="J45" s="52">
         <f>J26-J43-J44</f>
       </c>
-      <c r="K45" s="51">
+      <c r="K45" s="52">
         <f>K26-K43-K44</f>
       </c>
-      <c r="L45" s="51">
+      <c r="L45" s="52">
         <f>L26-L43-L44</f>
       </c>
-      <c r="M45" s="51">
+      <c r="M45" s="52">
         <f>M26-M43-M44</f>
       </c>
-      <c r="N45" s="51">
+      <c r="N45" s="52">
         <f>N26-N43-N44</f>
       </c>
-      <c r="O45" s="51">
+      <c r="O45" s="52">
         <f>O26-O43-O44</f>
       </c>
-      <c r="P45" s="51">
+      <c r="P45" s="52">
         <f>SUM(D45:O45)</f>
       </c>
     </row>
@@ -3470,43 +3476,43 @@
       <c r="P46" s="20"/>
     </row>
     <row r="47" ht="20" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B47" s="44" t="s">
-        <v>110</v>
-      </c>
-      <c r="D47" s="46">
+      <c r="B47" s="45" t="s">
+        <v>111</v>
+      </c>
+      <c r="D47" s="47">
         <f>D29*D4</f>
       </c>
-      <c r="E47" s="46">
+      <c r="E47" s="47">
         <f>E29*E4</f>
       </c>
-      <c r="F47" s="46">
+      <c r="F47" s="47">
         <f>F29*F4</f>
       </c>
-      <c r="G47" s="46">
+      <c r="G47" s="47">
         <f>G29*G4</f>
       </c>
-      <c r="H47" s="46">
+      <c r="H47" s="47">
         <f>H29*H4</f>
       </c>
-      <c r="I47" s="46">
+      <c r="I47" s="47">
         <f>I29*I4</f>
       </c>
-      <c r="J47" s="46">
+      <c r="J47" s="47">
         <f>J29*J4</f>
       </c>
-      <c r="K47" s="46">
+      <c r="K47" s="47">
         <f>K29*K4</f>
       </c>
-      <c r="L47" s="46">
+      <c r="L47" s="47">
         <f>L29*L4</f>
       </c>
-      <c r="M47" s="46">
+      <c r="M47" s="47">
         <f>M29*M4</f>
       </c>
-      <c r="N47" s="46">
+      <c r="N47" s="47">
         <f>N29*N4</f>
       </c>
-      <c r="O47" s="46">
+      <c r="O47" s="47">
         <f>O29*O4</f>
       </c>
       <c r="P47" s="25">
@@ -3514,96 +3520,96 @@
       </c>
     </row>
     <row r="48" ht="26" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B48" s="52" t="s">
-        <v>111</v>
-      </c>
-      <c r="C48" s="53" t="s">
+      <c r="B48" s="53" t="s">
         <v>112</v>
       </c>
-      <c r="D48" s="54">
+      <c r="C48" s="54" t="s">
+        <v>113</v>
+      </c>
+      <c r="D48" s="55">
         <f>D29+D31-D40-D47</f>
       </c>
-      <c r="E48" s="54">
+      <c r="E48" s="55">
         <f>E29+E31-E40-E47</f>
       </c>
-      <c r="F48" s="54">
+      <c r="F48" s="55">
         <f>F29+F31-F40-F47</f>
       </c>
-      <c r="G48" s="54">
+      <c r="G48" s="55">
         <f>G29+G31-G40-G47</f>
       </c>
-      <c r="H48" s="54">
+      <c r="H48" s="55">
         <f>H29+H31-H40-H47</f>
       </c>
-      <c r="I48" s="54">
+      <c r="I48" s="55">
         <f>I29+I31-I40-I47</f>
       </c>
-      <c r="J48" s="54">
+      <c r="J48" s="55">
         <f>J29+J31-J40-J47</f>
       </c>
-      <c r="K48" s="54">
+      <c r="K48" s="55">
         <f>K29+K31-K40-K47</f>
       </c>
-      <c r="L48" s="54">
+      <c r="L48" s="55">
         <f>L29+L31-L40-L47</f>
       </c>
-      <c r="M48" s="54">
+      <c r="M48" s="55">
         <f>M29+M31-M40-M47</f>
       </c>
-      <c r="N48" s="54">
+      <c r="N48" s="55">
         <f>N29+N31-N40-N47</f>
       </c>
-      <c r="O48" s="54">
+      <c r="O48" s="55">
         <f>O29+O31-O40-O47</f>
       </c>
-      <c r="P48" s="54">
+      <c r="P48" s="55">
         <f>SUM(D48:O48)</f>
       </c>
     </row>
     <row r="49" ht="28" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B49" s="52" t="s">
-        <v>113</v>
-      </c>
-      <c r="C49" s="53" t="s">
+      <c r="B49" s="53" t="s">
         <v>114</v>
       </c>
-      <c r="D49" s="54">
+      <c r="C49" s="54" t="s">
+        <v>115</v>
+      </c>
+      <c r="D49" s="55">
         <f>D48+D45</f>
       </c>
-      <c r="E49" s="54">
+      <c r="E49" s="55">
         <f>E48+E45</f>
       </c>
-      <c r="F49" s="54">
+      <c r="F49" s="55">
         <f>F48+F45</f>
       </c>
-      <c r="G49" s="54">
+      <c r="G49" s="55">
         <f>G48+G45</f>
       </c>
-      <c r="H49" s="54">
+      <c r="H49" s="55">
         <f>H48+H45</f>
       </c>
-      <c r="I49" s="54">
+      <c r="I49" s="55">
         <f>I48+I45</f>
       </c>
-      <c r="J49" s="54">
+      <c r="J49" s="55">
         <f>J48+J45</f>
       </c>
-      <c r="K49" s="54">
+      <c r="K49" s="55">
         <f>K48+K45</f>
       </c>
-      <c r="L49" s="54">
+      <c r="L49" s="55">
         <f>L48+L45</f>
       </c>
-      <c r="M49" s="54">
+      <c r="M49" s="55">
         <f>M48+M45</f>
       </c>
-      <c r="N49" s="54">
+      <c r="N49" s="55">
         <f>N48+N45</f>
       </c>
-      <c r="O49" s="54">
+      <c r="O49" s="55">
         <f>O48+O45</f>
       </c>
-      <c r="P49" s="54">
+      <c r="P49" s="55">
         <f>SUM(D49:O49)</f>
       </c>
     </row>
@@ -3626,66 +3632,66 @@
       <c r="P50" s="2"/>
     </row>
     <row r="51" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A51" s="55" t="s">
-        <v>115</v>
-      </c>
-      <c r="B51" s="55"/>
-      <c r="C51" s="55"/>
-      <c r="D51" s="55"/>
-      <c r="E51" s="55"/>
-      <c r="F51" s="55"/>
-      <c r="G51" s="55"/>
-      <c r="H51" s="55"/>
-      <c r="I51" s="55"/>
-      <c r="J51" s="55"/>
-      <c r="K51" s="55"/>
-      <c r="L51" s="55"/>
-      <c r="M51" s="55"/>
-      <c r="N51" s="55"/>
-      <c r="O51" s="55"/>
-      <c r="P51" s="55"/>
+      <c r="A51" s="56" t="s">
+        <v>116</v>
+      </c>
+      <c r="B51" s="56"/>
+      <c r="C51" s="56"/>
+      <c r="D51" s="56"/>
+      <c r="E51" s="56"/>
+      <c r="F51" s="56"/>
+      <c r="G51" s="56"/>
+      <c r="H51" s="56"/>
+      <c r="I51" s="56"/>
+      <c r="J51" s="56"/>
+      <c r="K51" s="56"/>
+      <c r="L51" s="56"/>
+      <c r="M51" s="56"/>
+      <c r="N51" s="56"/>
+      <c r="O51" s="56"/>
+      <c r="P51" s="56"/>
     </row>
     <row r="52" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B52" s="56" t="s">
-        <v>116</v>
-      </c>
-      <c r="C52" s="57" t="s">
+      <c r="B52" s="57" t="s">
         <v>117</v>
       </c>
-      <c r="D52" s="58">
+      <c r="C52" s="58" t="s">
+        <v>118</v>
+      </c>
+      <c r="D52" s="59">
         <f>D16</f>
       </c>
-      <c r="E52" s="58">
+      <c r="E52" s="59">
         <f>E16</f>
       </c>
-      <c r="F52" s="58">
+      <c r="F52" s="59">
         <f>F16</f>
       </c>
-      <c r="G52" s="58">
+      <c r="G52" s="59">
         <f>G16</f>
       </c>
-      <c r="H52" s="58">
+      <c r="H52" s="59">
         <f>H16</f>
       </c>
-      <c r="I52" s="58">
+      <c r="I52" s="59">
         <f>I16</f>
       </c>
-      <c r="J52" s="58">
+      <c r="J52" s="59">
         <f>J16</f>
       </c>
-      <c r="K52" s="58">
+      <c r="K52" s="59">
         <f>K16</f>
       </c>
-      <c r="L52" s="58">
+      <c r="L52" s="59">
         <f>L16</f>
       </c>
-      <c r="M52" s="58">
+      <c r="M52" s="59">
         <f>M16</f>
       </c>
-      <c r="N52" s="58">
+      <c r="N52" s="59">
         <f>N16</f>
       </c>
-      <c r="O52" s="58">
+      <c r="O52" s="59">
         <f>O16</f>
       </c>
       <c r="P52" s="25">
@@ -3693,46 +3699,46 @@
       </c>
     </row>
     <row r="53" ht="18" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B53" s="56" t="s">
-        <v>118</v>
-      </c>
-      <c r="C53" s="57" t="s">
+      <c r="B53" s="57" t="s">
         <v>119</v>
       </c>
-      <c r="D53" s="59">
+      <c r="C53" s="58" t="s">
+        <v>120</v>
+      </c>
+      <c r="D53" s="60">
         <f>(Configuración!$C$5/31)*D52</f>
       </c>
-      <c r="E53" s="59">
+      <c r="E53" s="60">
         <f>(Configuración!$C$5/28)*E52</f>
       </c>
-      <c r="F53" s="59">
+      <c r="F53" s="60">
         <f>(Configuración!$C$5/31)*F52</f>
       </c>
-      <c r="G53" s="59">
+      <c r="G53" s="60">
         <f>(Configuración!$C$5/30)*G52</f>
       </c>
-      <c r="H53" s="59">
+      <c r="H53" s="60">
         <f>(Configuración!$C$5/31)*H52</f>
       </c>
-      <c r="I53" s="59">
+      <c r="I53" s="60">
         <f>(Configuración!$C$5/30)*I52</f>
       </c>
-      <c r="J53" s="59">
+      <c r="J53" s="60">
         <f>(Configuración!$C$5/31)*J52</f>
       </c>
-      <c r="K53" s="59">
+      <c r="K53" s="60">
         <f>(Configuración!$C$5/31)*K52</f>
       </c>
-      <c r="L53" s="59">
+      <c r="L53" s="60">
         <f>(Configuración!$C$5/30)*L52</f>
       </c>
-      <c r="M53" s="59">
+      <c r="M53" s="60">
         <f>(Configuración!$C$5/31)*M52</f>
       </c>
-      <c r="N53" s="59">
+      <c r="N53" s="60">
         <f>(Configuración!$C$5/30)*N52</f>
       </c>
-      <c r="O53" s="59">
+      <c r="O53" s="60">
         <f>(Configuración!$C$5/31)*O52</f>
       </c>
       <c r="P53" s="25">
@@ -3740,96 +3746,96 @@
       </c>
     </row>
     <row r="54" ht="20" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B54" s="60" t="s">
-        <v>120</v>
-      </c>
-      <c r="C54" s="57" t="s">
+      <c r="B54" s="61" t="s">
         <v>121</v>
       </c>
-      <c r="D54" s="61">
-        <f>D53+D14*Configuración!$C$27+D15*Configuración!$C$28+D16*Configuración!$C$31</f>
-      </c>
-      <c r="E54" s="61">
-        <f>E53+E14*Configuración!$C$27+E15*Configuración!$C$28+E16*Configuración!$C$31</f>
-      </c>
-      <c r="F54" s="61">
-        <f>F53+F14*Configuración!$C$27+F15*Configuración!$C$28+F16*Configuración!$C$31</f>
-      </c>
-      <c r="G54" s="61">
-        <f>G53+G14*Configuración!$C$27+G15*Configuración!$C$28+G16*Configuración!$C$31</f>
-      </c>
-      <c r="H54" s="61">
-        <f>H53+H14*Configuración!$C$27+H15*Configuración!$C$28+H16*Configuración!$C$31</f>
-      </c>
-      <c r="I54" s="61">
-        <f>I53+I14*Configuración!$C$27+I15*Configuración!$C$28+I16*Configuración!$C$31</f>
-      </c>
-      <c r="J54" s="61">
-        <f>J53+J14*Configuración!$C$27+J15*Configuración!$C$28+J16*Configuración!$C$31</f>
-      </c>
-      <c r="K54" s="61">
-        <f>K53+K14*Configuración!$C$27+K15*Configuración!$C$28+K16*Configuración!$C$31</f>
-      </c>
-      <c r="L54" s="61">
-        <f>L53+L14*Configuración!$C$27+L15*Configuración!$C$28+L16*Configuración!$C$31</f>
-      </c>
-      <c r="M54" s="61">
-        <f>M53+M14*Configuración!$C$27+M15*Configuración!$C$28+M16*Configuración!$C$31</f>
-      </c>
-      <c r="N54" s="61">
-        <f>N53+N14*Configuración!$C$27+N15*Configuración!$C$28+N16*Configuración!$C$31</f>
-      </c>
-      <c r="O54" s="61">
-        <f>O53+O14*Configuración!$C$27+O15*Configuración!$C$28+O16*Configuración!$C$31</f>
-      </c>
-      <c r="P54" s="61">
+      <c r="C54" s="58" t="s">
+        <v>122</v>
+      </c>
+      <c r="D54" s="62">
+        <f>D53+D14*Configuración!$C$27+D15*Configuración!$C$28</f>
+      </c>
+      <c r="E54" s="62">
+        <f>E53+E14*Configuración!$C$27+E15*Configuración!$C$28</f>
+      </c>
+      <c r="F54" s="62">
+        <f>F53+F14*Configuración!$C$27+F15*Configuración!$C$28</f>
+      </c>
+      <c r="G54" s="62">
+        <f>G53+G14*Configuración!$C$27+G15*Configuración!$C$28</f>
+      </c>
+      <c r="H54" s="62">
+        <f>H53+H14*Configuración!$C$27+H15*Configuración!$C$28</f>
+      </c>
+      <c r="I54" s="62">
+        <f>I53+I14*Configuración!$C$27+I15*Configuración!$C$28</f>
+      </c>
+      <c r="J54" s="62">
+        <f>J53+J14*Configuración!$C$27+J15*Configuración!$C$28</f>
+      </c>
+      <c r="K54" s="62">
+        <f>K53+K14*Configuración!$C$27+K15*Configuración!$C$28</f>
+      </c>
+      <c r="L54" s="62">
+        <f>L53+L14*Configuración!$C$27+L15*Configuración!$C$28</f>
+      </c>
+      <c r="M54" s="62">
+        <f>M53+M14*Configuración!$C$27+M15*Configuración!$C$28</f>
+      </c>
+      <c r="N54" s="62">
+        <f>N53+N14*Configuración!$C$27+N15*Configuración!$C$28</f>
+      </c>
+      <c r="O54" s="62">
+        <f>O53+O14*Configuración!$C$27+O15*Configuración!$C$28</f>
+      </c>
+      <c r="P54" s="62">
         <f>SUM(D54:O54)</f>
       </c>
     </row>
     <row r="55" ht="22" customHeight="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B55" s="62" t="s">
-        <v>122</v>
-      </c>
-      <c r="C55" s="63" t="s">
+      <c r="B55" s="63" t="s">
         <v>123</v>
       </c>
-      <c r="D55" s="64">
+      <c r="C55" s="64" t="s">
+        <v>124</v>
+      </c>
+      <c r="D55" s="65">
         <f>D54*D4</f>
       </c>
-      <c r="E55" s="64">
+      <c r="E55" s="65">
         <f>E54*E4</f>
       </c>
-      <c r="F55" s="64">
+      <c r="F55" s="65">
         <f>F54*F4</f>
       </c>
-      <c r="G55" s="64">
+      <c r="G55" s="65">
         <f>G54*G4</f>
       </c>
-      <c r="H55" s="64">
+      <c r="H55" s="65">
         <f>H54*H4</f>
       </c>
-      <c r="I55" s="64">
+      <c r="I55" s="65">
         <f>I54*I4</f>
       </c>
-      <c r="J55" s="64">
+      <c r="J55" s="65">
         <f>J54*J4</f>
       </c>
-      <c r="K55" s="64">
+      <c r="K55" s="65">
         <f>K54*K4</f>
       </c>
-      <c r="L55" s="64">
+      <c r="L55" s="65">
         <f>L54*L4</f>
       </c>
-      <c r="M55" s="64">
+      <c r="M55" s="65">
         <f>M54*M4</f>
       </c>
-      <c r="N55" s="64">
+      <c r="N55" s="65">
         <f>N54*N4</f>
       </c>
-      <c r="O55" s="64">
+      <c r="O55" s="65">
         <f>O54*O4</f>
       </c>
-      <c r="P55" s="64">
+      <c r="P55" s="65">
         <f>SUM(D55:O55)</f>
       </c>
     </row>
@@ -3852,112 +3858,112 @@
       <c r="P56" s="2"/>
     </row>
     <row r="57" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A57" s="55" t="s">
-        <v>124</v>
-      </c>
-      <c r="B57" s="55"/>
-      <c r="C57" s="55"/>
-      <c r="D57" s="55"/>
-      <c r="E57" s="55"/>
-      <c r="F57" s="55"/>
-      <c r="G57" s="55"/>
-      <c r="H57" s="55"/>
-      <c r="I57" s="55"/>
-      <c r="J57" s="55"/>
-      <c r="K57" s="55"/>
-      <c r="L57" s="55"/>
-      <c r="M57" s="55"/>
-      <c r="N57" s="55"/>
-      <c r="O57" s="55"/>
-      <c r="P57" s="55"/>
+      <c r="A57" s="56" t="s">
+        <v>125</v>
+      </c>
+      <c r="B57" s="56"/>
+      <c r="C57" s="56"/>
+      <c r="D57" s="56"/>
+      <c r="E57" s="56"/>
+      <c r="F57" s="56"/>
+      <c r="G57" s="56"/>
+      <c r="H57" s="56"/>
+      <c r="I57" s="56"/>
+      <c r="J57" s="56"/>
+      <c r="K57" s="56"/>
+      <c r="L57" s="56"/>
+      <c r="M57" s="56"/>
+      <c r="N57" s="56"/>
+      <c r="O57" s="56"/>
+      <c r="P57" s="56"/>
     </row>
     <row r="58" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A58" s="65" t="s">
-        <v>125</v>
-      </c>
-      <c r="B58" s="65"/>
-      <c r="C58" s="65"/>
-      <c r="D58" s="65"/>
-      <c r="E58" s="65"/>
-      <c r="F58" s="65"/>
-      <c r="G58" s="65"/>
-      <c r="H58" s="65"/>
-      <c r="I58" s="65"/>
-      <c r="J58" s="65"/>
-      <c r="K58" s="65"/>
-      <c r="L58" s="65"/>
-      <c r="M58" s="65"/>
-      <c r="N58" s="66">
+      <c r="A58" s="66" t="s">
+        <v>126</v>
+      </c>
+      <c r="B58" s="66"/>
+      <c r="C58" s="66"/>
+      <c r="D58" s="66"/>
+      <c r="E58" s="66"/>
+      <c r="F58" s="66"/>
+      <c r="G58" s="66"/>
+      <c r="H58" s="66"/>
+      <c r="I58" s="66"/>
+      <c r="J58" s="66"/>
+      <c r="K58" s="66"/>
+      <c r="L58" s="66"/>
+      <c r="M58" s="66"/>
+      <c r="N58" s="67">
         <f>SUM(D54:O54)</f>
       </c>
-      <c r="O58" s="66"/>
-      <c r="P58" s="66"/>
+      <c r="O58" s="67"/>
+      <c r="P58" s="67"/>
     </row>
     <row r="59" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A59" s="65" t="s">
-        <v>126</v>
-      </c>
-      <c r="B59" s="65"/>
-      <c r="C59" s="65"/>
-      <c r="D59" s="65"/>
-      <c r="E59" s="65"/>
-      <c r="F59" s="65"/>
-      <c r="G59" s="65"/>
-      <c r="H59" s="65"/>
-      <c r="I59" s="65"/>
-      <c r="J59" s="65"/>
-      <c r="K59" s="65"/>
-      <c r="L59" s="65"/>
-      <c r="M59" s="65"/>
-      <c r="N59" s="66">
+      <c r="A59" s="66" t="s">
+        <v>127</v>
+      </c>
+      <c r="B59" s="66"/>
+      <c r="C59" s="66"/>
+      <c r="D59" s="66"/>
+      <c r="E59" s="66"/>
+      <c r="F59" s="66"/>
+      <c r="G59" s="66"/>
+      <c r="H59" s="66"/>
+      <c r="I59" s="66"/>
+      <c r="J59" s="66"/>
+      <c r="K59" s="66"/>
+      <c r="L59" s="66"/>
+      <c r="M59" s="66"/>
+      <c r="N59" s="67">
         <v>60100</v>
       </c>
-      <c r="O59" s="66"/>
-      <c r="P59" s="66"/>
+      <c r="O59" s="67"/>
+      <c r="P59" s="67"/>
     </row>
     <row r="60" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A60" s="65" t="s">
-        <v>127</v>
-      </c>
-      <c r="B60" s="65"/>
-      <c r="C60" s="65"/>
-      <c r="D60" s="65"/>
-      <c r="E60" s="65"/>
-      <c r="F60" s="65"/>
-      <c r="G60" s="65"/>
-      <c r="H60" s="65"/>
-      <c r="I60" s="65"/>
-      <c r="J60" s="65"/>
-      <c r="K60" s="65"/>
-      <c r="L60" s="65"/>
-      <c r="M60" s="65"/>
-      <c r="N60" s="66">
+      <c r="A60" s="66" t="s">
+        <v>128</v>
+      </c>
+      <c r="B60" s="66"/>
+      <c r="C60" s="66"/>
+      <c r="D60" s="66"/>
+      <c r="E60" s="66"/>
+      <c r="F60" s="66"/>
+      <c r="G60" s="66"/>
+      <c r="H60" s="66"/>
+      <c r="I60" s="66"/>
+      <c r="J60" s="66"/>
+      <c r="K60" s="66"/>
+      <c r="L60" s="66"/>
+      <c r="M60" s="66"/>
+      <c r="N60" s="67">
         <f>60100-SUM(D54:O54)</f>
       </c>
-      <c r="O60" s="66"/>
-      <c r="P60" s="66"/>
+      <c r="O60" s="67"/>
+      <c r="P60" s="67"/>
     </row>
     <row r="61" ht="30" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A61" s="67" t="s">
-        <v>128</v>
-      </c>
-      <c r="B61" s="67"/>
-      <c r="C61" s="67"/>
-      <c r="D61" s="67"/>
-      <c r="E61" s="67"/>
-      <c r="F61" s="67"/>
-      <c r="G61" s="67"/>
-      <c r="H61" s="67"/>
-      <c r="I61" s="67"/>
-      <c r="J61" s="67"/>
-      <c r="K61" s="67"/>
-      <c r="L61" s="67"/>
-      <c r="M61" s="67"/>
-      <c r="N61" s="68">
+      <c r="A61" s="68" t="s">
+        <v>129</v>
+      </c>
+      <c r="B61" s="68"/>
+      <c r="C61" s="68"/>
+      <c r="D61" s="68"/>
+      <c r="E61" s="68"/>
+      <c r="F61" s="68"/>
+      <c r="G61" s="68"/>
+      <c r="H61" s="68"/>
+      <c r="I61" s="68"/>
+      <c r="J61" s="68"/>
+      <c r="K61" s="68"/>
+      <c r="L61" s="68"/>
+      <c r="M61" s="68"/>
+      <c r="N61" s="69">
         <f>SUM(D55:O55)</f>
       </c>
-      <c r="O61" s="68"/>
-      <c r="P61" s="68"/>
+      <c r="O61" s="69"/>
+      <c r="P61" s="69"/>
     </row>
     <row r="62" ht="8" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" s="2"/>
@@ -3979,7 +3985,7 @@
     </row>
     <row r="63" ht="32" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B63" s="10"/>
       <c r="C63" s="10"/>
@@ -4016,88 +4022,88 @@
       <c r="P64" s="2"/>
     </row>
     <row r="65" ht="24" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A65" s="69" t="s">
-        <v>130</v>
-      </c>
-      <c r="B65" s="69"/>
-      <c r="C65" s="69"/>
-      <c r="D65" s="69"/>
-      <c r="E65" s="69"/>
-      <c r="F65" s="69"/>
-      <c r="G65" s="69"/>
-      <c r="H65" s="69"/>
-      <c r="I65" s="69"/>
-      <c r="J65" s="69"/>
-      <c r="K65" s="69"/>
-      <c r="L65" s="69"/>
-      <c r="M65" s="69"/>
-      <c r="N65" s="69"/>
-      <c r="O65" s="69"/>
-      <c r="P65" s="69"/>
+      <c r="A65" s="70" t="s">
+        <v>131</v>
+      </c>
+      <c r="B65" s="70"/>
+      <c r="C65" s="70"/>
+      <c r="D65" s="70"/>
+      <c r="E65" s="70"/>
+      <c r="F65" s="70"/>
+      <c r="G65" s="70"/>
+      <c r="H65" s="70"/>
+      <c r="I65" s="70"/>
+      <c r="J65" s="70"/>
+      <c r="K65" s="70"/>
+      <c r="L65" s="70"/>
+      <c r="M65" s="70"/>
+      <c r="N65" s="70"/>
+      <c r="O65" s="70"/>
+      <c r="P65" s="70"/>
     </row>
     <row r="66" ht="30" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A66" s="70" t="s">
-        <v>131</v>
-      </c>
-      <c r="B66" s="70"/>
-      <c r="C66" s="70"/>
-      <c r="D66" s="70"/>
-      <c r="E66" s="70"/>
-      <c r="F66" s="70"/>
-      <c r="G66" s="70"/>
-      <c r="H66" s="70"/>
-      <c r="I66" s="70"/>
-      <c r="J66" s="70"/>
-      <c r="K66" s="70"/>
-      <c r="L66" s="70"/>
-      <c r="M66" s="70"/>
-      <c r="N66" s="70"/>
-      <c r="O66" s="70"/>
-      <c r="P66" s="71">
+      <c r="A66" s="71" t="s">
+        <v>132</v>
+      </c>
+      <c r="B66" s="71"/>
+      <c r="C66" s="71"/>
+      <c r="D66" s="71"/>
+      <c r="E66" s="71"/>
+      <c r="F66" s="71"/>
+      <c r="G66" s="71"/>
+      <c r="H66" s="71"/>
+      <c r="I66" s="71"/>
+      <c r="J66" s="71"/>
+      <c r="K66" s="71"/>
+      <c r="L66" s="71"/>
+      <c r="M66" s="71"/>
+      <c r="N66" s="71"/>
+      <c r="O66" s="71"/>
+      <c r="P66" s="72">
         <f>SUM(D29:O29)+SUM(D31:O31)+SUM(D26:O26)</f>
       </c>
     </row>
     <row r="67" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A67" s="72" t="s">
-        <v>132</v>
-      </c>
-      <c r="B67" s="72"/>
-      <c r="C67" s="72"/>
-      <c r="D67" s="72"/>
-      <c r="E67" s="72"/>
-      <c r="F67" s="72"/>
-      <c r="G67" s="72"/>
-      <c r="H67" s="72"/>
-      <c r="I67" s="72"/>
-      <c r="J67" s="72"/>
-      <c r="K67" s="72"/>
-      <c r="L67" s="72"/>
-      <c r="M67" s="72"/>
-      <c r="N67" s="72"/>
-      <c r="O67" s="72"/>
-      <c r="P67" s="73">
+      <c r="A67" s="73" t="s">
+        <v>133</v>
+      </c>
+      <c r="B67" s="73"/>
+      <c r="C67" s="73"/>
+      <c r="D67" s="73"/>
+      <c r="E67" s="73"/>
+      <c r="F67" s="73"/>
+      <c r="G67" s="73"/>
+      <c r="H67" s="73"/>
+      <c r="I67" s="73"/>
+      <c r="J67" s="73"/>
+      <c r="K67" s="73"/>
+      <c r="L67" s="73"/>
+      <c r="M67" s="73"/>
+      <c r="N67" s="73"/>
+      <c r="O67" s="73"/>
+      <c r="P67" s="74">
         <f>Configuración!$C$5*12</f>
       </c>
     </row>
     <row r="68" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A68" s="74" t="s">
-        <v>133</v>
-      </c>
-      <c r="B68" s="74"/>
-      <c r="C68" s="74"/>
-      <c r="D68" s="74"/>
-      <c r="E68" s="74"/>
-      <c r="F68" s="74"/>
-      <c r="G68" s="74"/>
-      <c r="H68" s="74"/>
-      <c r="I68" s="74"/>
-      <c r="J68" s="74"/>
-      <c r="K68" s="74"/>
-      <c r="L68" s="74"/>
-      <c r="M68" s="74"/>
-      <c r="N68" s="74"/>
-      <c r="O68" s="74"/>
-      <c r="P68" s="75">
+      <c r="A68" s="75" t="s">
+        <v>134</v>
+      </c>
+      <c r="B68" s="75"/>
+      <c r="C68" s="75"/>
+      <c r="D68" s="75"/>
+      <c r="E68" s="75"/>
+      <c r="F68" s="75"/>
+      <c r="G68" s="75"/>
+      <c r="H68" s="75"/>
+      <c r="I68" s="75"/>
+      <c r="J68" s="75"/>
+      <c r="K68" s="75"/>
+      <c r="L68" s="75"/>
+      <c r="M68" s="75"/>
+      <c r="N68" s="75"/>
+      <c r="O68" s="75"/>
+      <c r="P68" s="76">
         <f>(SUM(D29:O29)+SUM(D31:O31)+SUM(D26:O26))-(Configuración!$C$5*12)</f>
       </c>
     </row>
@@ -4120,68 +4126,68 @@
       <c r="P69" s="20"/>
     </row>
     <row r="70" ht="30" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A70" s="76" t="s">
+      <c r="A70" s="77" t="s">
+        <v>135</v>
+      </c>
+      <c r="B70" s="77"/>
+      <c r="C70" s="77"/>
+      <c r="D70" s="77"/>
+      <c r="E70" s="77"/>
+      <c r="F70" s="77"/>
+      <c r="G70" s="77"/>
+      <c r="H70" s="77"/>
+      <c r="I70" s="77"/>
+      <c r="J70" s="77"/>
+      <c r="K70" s="77"/>
+      <c r="L70" s="77"/>
+      <c r="M70" s="77"/>
+      <c r="N70" s="77"/>
+      <c r="O70" s="77"/>
+      <c r="P70" s="78">
+        <f>SUM(D49:O49)</f>
+      </c>
+    </row>
+    <row r="71" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A71" s="73" t="s">
+        <v>136</v>
+      </c>
+      <c r="B71" s="73"/>
+      <c r="C71" s="73"/>
+      <c r="D71" s="73"/>
+      <c r="E71" s="73"/>
+      <c r="F71" s="73"/>
+      <c r="G71" s="73"/>
+      <c r="H71" s="73"/>
+      <c r="I71" s="73"/>
+      <c r="J71" s="73"/>
+      <c r="K71" s="73"/>
+      <c r="L71" s="73"/>
+      <c r="M71" s="73"/>
+      <c r="N71" s="73"/>
+      <c r="O71" s="73"/>
+      <c r="P71" s="74">
+        <f>Configuración!$C$5*12-(Configuración!$C$5*12+Configuración!$C$7*12)*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)-Configuración!$C$5*12*Configuración!$C$18</f>
+      </c>
+    </row>
+    <row r="72" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A72" s="75" t="s">
         <v>134</v>
       </c>
-      <c r="B70" s="76"/>
-      <c r="C70" s="76"/>
-      <c r="D70" s="76"/>
-      <c r="E70" s="76"/>
-      <c r="F70" s="76"/>
-      <c r="G70" s="76"/>
-      <c r="H70" s="76"/>
-      <c r="I70" s="76"/>
-      <c r="J70" s="76"/>
-      <c r="K70" s="76"/>
-      <c r="L70" s="76"/>
-      <c r="M70" s="76"/>
-      <c r="N70" s="76"/>
-      <c r="O70" s="76"/>
-      <c r="P70" s="77">
-        <f>SUM(D49:O49)</f>
-      </c>
-    </row>
-    <row r="71" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A71" s="72" t="s">
-        <v>135</v>
-      </c>
-      <c r="B71" s="72"/>
-      <c r="C71" s="72"/>
-      <c r="D71" s="72"/>
-      <c r="E71" s="72"/>
-      <c r="F71" s="72"/>
-      <c r="G71" s="72"/>
-      <c r="H71" s="72"/>
-      <c r="I71" s="72"/>
-      <c r="J71" s="72"/>
-      <c r="K71" s="72"/>
-      <c r="L71" s="72"/>
-      <c r="M71" s="72"/>
-      <c r="N71" s="72"/>
-      <c r="O71" s="72"/>
-      <c r="P71" s="73">
-        <f>Configuración!$C$5*12-(Configuración!$C$5*12+Configuración!$C$7*12)*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)-Configuración!$C$5*12*Configuración!$C$18</f>
-      </c>
-    </row>
-    <row r="72" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A72" s="74" t="s">
-        <v>133</v>
-      </c>
-      <c r="B72" s="74"/>
-      <c r="C72" s="74"/>
-      <c r="D72" s="74"/>
-      <c r="E72" s="74"/>
-      <c r="F72" s="74"/>
-      <c r="G72" s="74"/>
-      <c r="H72" s="74"/>
-      <c r="I72" s="74"/>
-      <c r="J72" s="74"/>
-      <c r="K72" s="74"/>
-      <c r="L72" s="74"/>
-      <c r="M72" s="74"/>
-      <c r="N72" s="74"/>
-      <c r="O72" s="74"/>
-      <c r="P72" s="75">
+      <c r="B72" s="75"/>
+      <c r="C72" s="75"/>
+      <c r="D72" s="75"/>
+      <c r="E72" s="75"/>
+      <c r="F72" s="75"/>
+      <c r="G72" s="75"/>
+      <c r="H72" s="75"/>
+      <c r="I72" s="75"/>
+      <c r="J72" s="75"/>
+      <c r="K72" s="75"/>
+      <c r="L72" s="75"/>
+      <c r="M72" s="75"/>
+      <c r="N72" s="75"/>
+      <c r="O72" s="75"/>
+      <c r="P72" s="76">
         <f>(SUM(D49:O49))-(Configuración!$C$5*12-(Configuración!$C$5*12+Configuración!$C$7*12)*(Configuración!$C$12+Configuración!$C$13+Configuración!$C$15)-Configuración!$C$5*12*Configuración!$C$18)</f>
       </c>
     </row>

</xml_diff>

<commit_message>
Pre-carga todos los datos reales Ene–May desde Calculo_sueldo_mes.xlsx
Arrays de 12 meses para TUR/NOC/FRI/DES/DESF/DIAF/HEX/HEXF/DIETA
con los valores exactos extraídos de la calculadora del usuario.
Jun–Dic quedan a cero para rellenar cuando estén disponibles.

https://claude.ai/code/session_01WLGGf5vt4LjNM5wLNiuW4q
</commit_message>
<xml_diff>
--- a/calculadora-nomina-v3.xlsx
+++ b/calculadora-nomina-v3.xlsx
@@ -2036,7 +2036,7 @@
         <v>0</v>
       </c>
       <c r="H9" s="26">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I9" s="26">
         <v>0</v>
@@ -2083,7 +2083,7 @@
         <v>0</v>
       </c>
       <c r="H10" s="26">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I10" s="26">
         <v>0</v>
@@ -2118,19 +2118,19 @@
         <v>68</v>
       </c>
       <c r="D11" s="26">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E11" s="26">
         <v>16</v>
       </c>
       <c r="F11" s="26">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G11" s="26">
         <v>0</v>
       </c>
       <c r="H11" s="26">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="I11" s="26">
         <v>0</v>
@@ -2259,19 +2259,19 @@
         <v>76</v>
       </c>
       <c r="D14" s="26">
-        <v>0</v>
+        <v>9.23</v>
       </c>
       <c r="E14" s="26">
-        <v>20.5</v>
+        <v>22.48</v>
       </c>
       <c r="F14" s="26">
-        <v>0</v>
+        <v>24.2</v>
       </c>
       <c r="G14" s="26">
-        <v>0</v>
+        <v>8.48</v>
       </c>
       <c r="H14" s="26">
-        <v>0</v>
+        <v>27.98</v>
       </c>
       <c r="I14" s="26">
         <v>0</v>
@@ -2306,19 +2306,19 @@
         <v>76</v>
       </c>
       <c r="D15" s="26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" s="26">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F15" s="26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" s="26">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="H15" s="26">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="I15" s="26">
         <v>0</v>
@@ -2356,7 +2356,7 @@
         <v>0</v>
       </c>
       <c r="E16" s="26">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F16" s="26">
         <v>0</v>
@@ -2400,19 +2400,19 @@
         <v>81</v>
       </c>
       <c r="D17" s="26">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="E17" s="26">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="F17" s="26">
-        <v>0</v>
+        <v>21.67</v>
       </c>
       <c r="G17" s="26">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H17" s="26">
-        <v>0</v>
+        <v>44.5</v>
       </c>
       <c r="I17" s="26">
         <v>0</v>
@@ -2447,19 +2447,19 @@
         <v>41</v>
       </c>
       <c r="D18" s="26">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E18" s="26">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="F18" s="26">
-        <v>0</v>
+        <v>6.67</v>
       </c>
       <c r="G18" s="26">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H18" s="26">
-        <v>0</v>
+        <v>44.5</v>
       </c>
       <c r="I18" s="26">
         <v>0</v>
@@ -2532,19 +2532,19 @@
         <v>85</v>
       </c>
       <c r="D21" s="6">
-        <v>0</v>
+        <v>286.56</v>
       </c>
       <c r="E21" s="6">
         <v>764.16</v>
       </c>
       <c r="F21" s="6">
-        <v>0</v>
+        <v>692.52</v>
       </c>
       <c r="G21" s="6">
-        <v>0</v>
+        <v>286.56</v>
       </c>
       <c r="H21" s="6">
-        <v>0</v>
+        <v>1098.48</v>
       </c>
       <c r="I21" s="6">
         <v>0</v>

</xml_diff>